<commit_message>
fix(requisiciones): recuadros de sellos en la plantilla y área de impresión completa
Los recuadros "SELLO UNIDAD" eran cuadros de texto flotantes que ExcelJS no conserva:
se dibujan ahora como celdas combinadas con borde punteado (izquierdo vacío, derecho
con la marca de agua) y el área de impresión llega hasta la fila 89.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/requisiciones_plantilla.xlsx
+++ b/requisiciones_plantilla.xlsx
@@ -10,14 +10,14 @@
     <sheet sheetId="44" name="GENERAL" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'GENERAL'!$A1:$K77</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'GENERAL'!$A1:$K89</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="90">
   <si>
     <t>SERVICIOS DE SALUD DEL ESTADO DE QUERÉTARO</t>
   </si>
@@ -295,6 +295,10 @@
   <si>
     <t>RECIBE: NOMBRE COMPLETO Y FIRMA</t>
   </si>
+  <si>
+    <t xml:space="preserve">SELLO
+UNIDAD</t>
+  </si>
 </sst>
 </file>
 
@@ -305,7 +309,7 @@
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy;@"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -416,6 +420,11 @@
       <sz val="10"/>
       <name val="Arial Nova"/>
     </font>
+    <font>
+      <color rgb="FFF9F9F9"/>
+      <sz val="138"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -443,7 +452,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -747,11 +756,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="dotted">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="dotted">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="dotted">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -1068,17 +1097,27 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -1089,8 +1128,8 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -2887,206 +2926,208 @@
       <c r="L75" s="96"/>
     </row>
     <row r="76" ht="20.25" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="83"/>
-      <c r="B76" s="83"/>
-      <c r="C76" s="83"/>
+      <c r="A76" s="98"/>
+      <c r="B76" s="98"/>
+      <c r="C76" s="98"/>
       <c r="D76" s="83"/>
       <c r="E76" s="83"/>
-      <c r="F76" s="98"/>
-      <c r="G76" s="99"/>
-      <c r="H76" s="99"/>
-      <c r="I76" s="99"/>
-      <c r="J76" s="99"/>
-      <c r="K76" s="100"/>
-      <c r="L76" s="101"/>
+      <c r="F76" s="99"/>
+      <c r="G76" s="100"/>
+      <c r="H76" s="101"/>
+      <c r="I76" s="101"/>
+      <c r="J76" s="101"/>
+      <c r="K76" s="102"/>
+      <c r="L76" s="103"/>
     </row>
     <row r="77" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="2"/>
-      <c r="B77" s="102"/>
-      <c r="C77" s="102"/>
-      <c r="D77" s="102"/>
-      <c r="E77" s="102"/>
+      <c r="A77" s="104"/>
+      <c r="B77" s="104"/>
+      <c r="C77" s="104"/>
+      <c r="D77" s="105"/>
+      <c r="E77" s="105"/>
       <c r="F77" s="2"/>
-      <c r="G77" s="103"/>
-      <c r="H77" s="103"/>
-      <c r="I77" s="103"/>
-      <c r="J77" s="103"/>
-      <c r="K77" s="2"/>
+      <c r="G77" s="106"/>
+      <c r="H77" s="107" t="s">
+        <v>89</v>
+      </c>
+      <c r="I77" s="107"/>
+      <c r="J77" s="107"/>
+      <c r="K77" s="107"/>
       <c r="L77" s="2"/>
     </row>
     <row r="78" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="2"/>
-      <c r="B78" s="2"/>
-      <c r="C78" s="2"/>
+      <c r="A78" s="104"/>
+      <c r="B78" s="104"/>
+      <c r="C78" s="104"/>
       <c r="D78" s="2"/>
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
-      <c r="G78" s="103"/>
-      <c r="H78" s="103"/>
-      <c r="I78" s="103"/>
-      <c r="J78" s="103"/>
-      <c r="K78" s="2"/>
+      <c r="G78" s="106"/>
+      <c r="H78" s="107"/>
+      <c r="I78" s="107"/>
+      <c r="J78" s="107"/>
+      <c r="K78" s="107"/>
       <c r="L78" s="2"/>
     </row>
     <row r="79" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="2"/>
-      <c r="B79" s="2"/>
-      <c r="C79" s="2"/>
+      <c r="A79" s="104"/>
+      <c r="B79" s="104"/>
+      <c r="C79" s="104"/>
       <c r="D79" s="2"/>
       <c r="E79" s="2"/>
       <c r="F79" s="2"/>
-      <c r="G79" s="103"/>
-      <c r="H79" s="103"/>
-      <c r="I79" s="103"/>
-      <c r="J79" s="103"/>
-      <c r="K79" s="2"/>
+      <c r="G79" s="106"/>
+      <c r="H79" s="107"/>
+      <c r="I79" s="107"/>
+      <c r="J79" s="107"/>
+      <c r="K79" s="107"/>
       <c r="L79" s="2"/>
     </row>
     <row r="80" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="2"/>
-      <c r="B80" s="2"/>
-      <c r="C80" s="2"/>
+      <c r="A80" s="104"/>
+      <c r="B80" s="104"/>
+      <c r="C80" s="104"/>
       <c r="D80" s="2"/>
       <c r="E80" s="2"/>
       <c r="F80" s="2"/>
-      <c r="G80" s="103"/>
-      <c r="H80" s="103"/>
-      <c r="I80" s="103"/>
-      <c r="J80" s="103"/>
-      <c r="K80" s="2"/>
+      <c r="G80" s="106"/>
+      <c r="H80" s="107"/>
+      <c r="I80" s="107"/>
+      <c r="J80" s="107"/>
+      <c r="K80" s="107"/>
       <c r="L80" s="2"/>
     </row>
     <row r="81" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="2"/>
-      <c r="B81" s="2"/>
-      <c r="C81" s="2"/>
+      <c r="A81" s="104"/>
+      <c r="B81" s="104"/>
+      <c r="C81" s="104"/>
       <c r="D81" s="2"/>
       <c r="E81" s="2"/>
       <c r="F81" s="2"/>
-      <c r="G81" s="103"/>
-      <c r="H81" s="103"/>
-      <c r="I81" s="103"/>
-      <c r="J81" s="103"/>
-      <c r="K81" s="2"/>
+      <c r="G81" s="106"/>
+      <c r="H81" s="107"/>
+      <c r="I81" s="107"/>
+      <c r="J81" s="107"/>
+      <c r="K81" s="107"/>
       <c r="L81" s="2"/>
     </row>
     <row r="82" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="2"/>
-      <c r="B82" s="2"/>
-      <c r="C82" s="2"/>
+      <c r="A82" s="104"/>
+      <c r="B82" s="104"/>
+      <c r="C82" s="104"/>
       <c r="D82" s="2"/>
       <c r="E82" s="2"/>
       <c r="F82" s="2"/>
-      <c r="G82" s="103"/>
-      <c r="H82" s="103"/>
-      <c r="I82" s="103"/>
-      <c r="J82" s="103"/>
-      <c r="K82" s="2"/>
+      <c r="G82" s="106"/>
+      <c r="H82" s="107"/>
+      <c r="I82" s="107"/>
+      <c r="J82" s="107"/>
+      <c r="K82" s="107"/>
       <c r="L82" s="2"/>
     </row>
     <row r="83" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="2"/>
-      <c r="B83" s="2"/>
-      <c r="C83" s="2"/>
+      <c r="A83" s="104"/>
+      <c r="B83" s="104"/>
+      <c r="C83" s="104"/>
       <c r="D83" s="2"/>
       <c r="E83" s="2"/>
       <c r="F83" s="2"/>
-      <c r="G83" s="103"/>
-      <c r="H83" s="103"/>
-      <c r="I83" s="103"/>
-      <c r="J83" s="103"/>
-      <c r="K83" s="2"/>
+      <c r="G83" s="106"/>
+      <c r="H83" s="107"/>
+      <c r="I83" s="107"/>
+      <c r="J83" s="107"/>
+      <c r="K83" s="107"/>
       <c r="L83" s="2"/>
     </row>
     <row r="84" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="2"/>
-      <c r="B84" s="2"/>
-      <c r="C84" s="2"/>
+      <c r="A84" s="104"/>
+      <c r="B84" s="104"/>
+      <c r="C84" s="104"/>
       <c r="D84" s="2"/>
       <c r="E84" s="2"/>
       <c r="F84" s="2"/>
-      <c r="G84" s="103"/>
-      <c r="H84" s="103"/>
-      <c r="I84" s="103"/>
-      <c r="J84" s="103"/>
-      <c r="K84" s="2"/>
+      <c r="G84" s="106"/>
+      <c r="H84" s="107"/>
+      <c r="I84" s="107"/>
+      <c r="J84" s="107"/>
+      <c r="K84" s="107"/>
       <c r="L84" s="2"/>
     </row>
     <row r="85" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="2"/>
-      <c r="B85" s="2"/>
-      <c r="C85" s="2"/>
+      <c r="A85" s="104"/>
+      <c r="B85" s="104"/>
+      <c r="C85" s="104"/>
       <c r="D85" s="2"/>
       <c r="E85" s="2"/>
       <c r="F85" s="2"/>
-      <c r="G85" s="103"/>
-      <c r="H85" s="103"/>
-      <c r="I85" s="103"/>
-      <c r="J85" s="103"/>
-      <c r="K85" s="2"/>
+      <c r="G85" s="106"/>
+      <c r="H85" s="107"/>
+      <c r="I85" s="107"/>
+      <c r="J85" s="107"/>
+      <c r="K85" s="107"/>
       <c r="L85" s="2"/>
     </row>
     <row r="86" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="2"/>
-      <c r="B86" s="2"/>
-      <c r="C86" s="2"/>
+      <c r="A86" s="104"/>
+      <c r="B86" s="104"/>
+      <c r="C86" s="104"/>
       <c r="D86" s="2"/>
       <c r="E86" s="2"/>
       <c r="F86" s="2"/>
-      <c r="G86" s="103"/>
-      <c r="H86" s="103"/>
-      <c r="I86" s="103"/>
-      <c r="J86" s="103"/>
-      <c r="K86" s="2"/>
+      <c r="G86" s="106"/>
+      <c r="H86" s="107"/>
+      <c r="I86" s="107"/>
+      <c r="J86" s="107"/>
+      <c r="K86" s="107"/>
       <c r="L86" s="2"/>
     </row>
     <row r="87" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="2"/>
-      <c r="B87" s="2"/>
-      <c r="C87" s="2"/>
+      <c r="A87" s="104"/>
+      <c r="B87" s="104"/>
+      <c r="C87" s="104"/>
       <c r="D87" s="2"/>
       <c r="E87" s="2"/>
       <c r="F87" s="2"/>
-      <c r="G87" s="103"/>
-      <c r="H87" s="103"/>
-      <c r="I87" s="103"/>
-      <c r="J87" s="103"/>
-      <c r="K87" s="2"/>
+      <c r="G87" s="106"/>
+      <c r="H87" s="107"/>
+      <c r="I87" s="107"/>
+      <c r="J87" s="107"/>
+      <c r="K87" s="107"/>
       <c r="L87" s="2"/>
     </row>
     <row r="88" ht="30" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A88" s="2"/>
-      <c r="B88" s="2"/>
-      <c r="C88" s="2"/>
+      <c r="A88" s="104"/>
+      <c r="B88" s="104"/>
+      <c r="C88" s="104"/>
       <c r="D88" s="2"/>
       <c r="E88" s="2"/>
       <c r="F88" s="2"/>
-      <c r="G88" s="103"/>
-      <c r="H88" s="103"/>
-      <c r="I88" s="103"/>
-      <c r="J88" s="103"/>
-      <c r="K88" s="2"/>
+      <c r="G88" s="106"/>
+      <c r="H88" s="107"/>
+      <c r="I88" s="107"/>
+      <c r="J88" s="107"/>
+      <c r="K88" s="107"/>
       <c r="L88" s="2"/>
     </row>
     <row r="89" ht="30" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A89" s="2"/>
-      <c r="B89" s="2"/>
-      <c r="C89" s="2"/>
+      <c r="A89" s="104"/>
+      <c r="B89" s="104"/>
+      <c r="C89" s="104"/>
       <c r="D89" s="2"/>
       <c r="E89" s="2"/>
       <c r="F89" s="2"/>
       <c r="G89" s="2"/>
-      <c r="H89" s="104"/>
-      <c r="I89" s="2"/>
-      <c r="J89" s="2"/>
-      <c r="K89" s="2"/>
+      <c r="H89" s="107"/>
+      <c r="I89" s="107"/>
+      <c r="J89" s="107"/>
+      <c r="K89" s="107"/>
       <c r="L89" s="2"/>
     </row>
     <row r="90" spans="13:17" x14ac:dyDescent="0.25"/>
     <row r="91" spans="13:17" x14ac:dyDescent="0.25"/>
     <row r="92" spans="13:17" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="184">
+  <mergeCells count="185">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A3:K3"/>
@@ -3270,7 +3311,8 @@
     <mergeCell ref="A75:C75"/>
     <mergeCell ref="H75:K75"/>
     <mergeCell ref="A76:C76"/>
-    <mergeCell ref="B77:C77"/>
+    <mergeCell ref="A77:C89"/>
+    <mergeCell ref="H77:K89"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.2362204724409449" right="0.2362204724409449" top="0.7480314960629921" bottom="0.7480314960629921" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
feat(requisiciones): más de 2 lotes por biológico en el Excel y bordes faltantes
- Un biológico con 3 o más lotes agrega renglones a ese biológico y baja el pie, las
  firmas y los recuadros de sellos; sigue en una página Carta.
- Plantilla: borde inferior en el último biológico (celdas combinadas) y borde completo
  en los recuadros de sellos (ExcelJS guarda un solo estilo por región combinada).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/requisiciones_plantilla.xlsx
+++ b/requisiciones_plantilla.xlsx
@@ -452,7 +452,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="27">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -724,7 +724,9 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -735,7 +737,52 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -766,11 +813,15 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="dotted">
+        <color rgb="FF000000"/>
+      </left>
       <right style="dotted">
         <color rgb="FF000000"/>
       </right>
-      <top/>
+      <top style="dotted">
+        <color rgb="FF000000"/>
+      </top>
       <bottom style="dotted">
         <color rgb="FF000000"/>
       </bottom>
@@ -780,7 +831,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -958,19 +1009,28 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="12" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1058,7 +1118,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1070,7 +1130,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -1093,11 +1153,11 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1106,17 +1166,17 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1128,7 +1188,7 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -2593,534 +2653,534 @@
       <c r="C54" s="58" t="s">
         <v>76</v>
       </c>
-      <c r="D54" s="38" t="s">
+      <c r="D54" s="59" t="s">
         <v>31</v>
       </c>
-      <c r="E54" s="39" t="s">
+      <c r="E54" s="60" t="s">
         <v>32</v>
       </c>
-      <c r="F54" s="40"/>
-      <c r="G54" s="59"/>
-      <c r="H54" s="59"/>
+      <c r="F54" s="61"/>
+      <c r="G54" s="62"/>
+      <c r="H54" s="62"/>
       <c r="I54" s="43"/>
       <c r="J54" s="44"/>
-      <c r="K54" s="60"/>
+      <c r="K54" s="63"/>
       <c r="L54" s="1"/>
     </row>
     <row r="55" ht="26.25" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="56"/>
       <c r="B55" s="57"/>
       <c r="C55" s="58"/>
-      <c r="D55" s="38"/>
-      <c r="E55" s="39"/>
-      <c r="F55" s="40"/>
+      <c r="D55" s="59"/>
+      <c r="E55" s="60"/>
+      <c r="F55" s="61"/>
       <c r="G55" s="47"/>
       <c r="H55" s="47"/>
       <c r="I55" s="48"/>
       <c r="J55" s="49"/>
-      <c r="K55" s="60"/>
+      <c r="K55" s="63"/>
       <c r="L55" s="1"/>
     </row>
     <row r="56" ht="25.5" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="61"/>
-      <c r="B56" s="62" t="s">
+      <c r="A56" s="64"/>
+      <c r="B56" s="65" t="s">
         <v>77</v>
       </c>
-      <c r="C56" s="62"/>
-      <c r="D56" s="62"/>
-      <c r="E56" s="62"/>
-      <c r="F56" s="62"/>
-      <c r="G56" s="62"/>
-      <c r="H56" s="62"/>
-      <c r="I56" s="62"/>
-      <c r="J56" s="62"/>
-      <c r="K56" s="63"/>
+      <c r="C56" s="65"/>
+      <c r="D56" s="65"/>
+      <c r="E56" s="65"/>
+      <c r="F56" s="65"/>
+      <c r="G56" s="65"/>
+      <c r="H56" s="65"/>
+      <c r="I56" s="65"/>
+      <c r="J56" s="65"/>
+      <c r="K56" s="66"/>
       <c r="L56" s="55"/>
     </row>
     <row r="57" ht="25.5" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="64"/>
-      <c r="B57" s="65"/>
-      <c r="C57" s="66"/>
-      <c r="D57" s="67"/>
-      <c r="E57" s="67"/>
-      <c r="F57" s="67"/>
-      <c r="G57" s="68"/>
-      <c r="H57" s="68"/>
-      <c r="I57" s="69"/>
-      <c r="J57" s="70"/>
-      <c r="K57" s="71"/>
+      <c r="A57" s="67"/>
+      <c r="B57" s="68"/>
+      <c r="C57" s="69"/>
+      <c r="D57" s="70"/>
+      <c r="E57" s="70"/>
+      <c r="F57" s="70"/>
+      <c r="G57" s="71"/>
+      <c r="H57" s="71"/>
+      <c r="I57" s="72"/>
+      <c r="J57" s="73"/>
+      <c r="K57" s="74"/>
       <c r="L57" s="8"/>
     </row>
     <row r="58" ht="25.5" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="64"/>
+      <c r="A58" s="67"/>
       <c r="B58" s="8"/>
-      <c r="C58" s="72" t="s">
+      <c r="C58" s="75" t="s">
         <v>78</v>
       </c>
-      <c r="D58" s="73"/>
-      <c r="E58" s="69"/>
-      <c r="F58" s="67"/>
-      <c r="G58" s="72" t="s">
+      <c r="D58" s="76"/>
+      <c r="E58" s="72"/>
+      <c r="F58" s="70"/>
+      <c r="G58" s="75" t="s">
         <v>79</v>
       </c>
-      <c r="H58" s="72"/>
-      <c r="I58" s="74"/>
-      <c r="J58" s="70"/>
-      <c r="K58" s="71"/>
+      <c r="H58" s="75"/>
+      <c r="I58" s="77"/>
+      <c r="J58" s="73"/>
+      <c r="K58" s="74"/>
       <c r="L58" s="8"/>
     </row>
     <row r="59" ht="25.5" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="64"/>
-      <c r="B59" s="65"/>
-      <c r="C59" s="66"/>
-      <c r="D59" s="67"/>
-      <c r="E59" s="67"/>
-      <c r="F59" s="67"/>
-      <c r="G59" s="68"/>
-      <c r="H59" s="68"/>
-      <c r="I59" s="69"/>
-      <c r="J59" s="70"/>
-      <c r="K59" s="71"/>
+      <c r="A59" s="67"/>
+      <c r="B59" s="68"/>
+      <c r="C59" s="69"/>
+      <c r="D59" s="70"/>
+      <c r="E59" s="70"/>
+      <c r="F59" s="70"/>
+      <c r="G59" s="71"/>
+      <c r="H59" s="71"/>
+      <c r="I59" s="72"/>
+      <c r="J59" s="73"/>
+      <c r="K59" s="74"/>
       <c r="L59" s="8"/>
     </row>
     <row r="60" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="75" t="s">
+      <c r="A60" s="78" t="s">
         <v>80</v>
       </c>
-      <c r="B60" s="75"/>
-      <c r="C60" s="75"/>
-      <c r="D60" s="75"/>
-      <c r="E60" s="75"/>
-      <c r="F60" s="75"/>
-      <c r="G60" s="75"/>
-      <c r="H60" s="75"/>
-      <c r="I60" s="75"/>
-      <c r="J60" s="75"/>
-      <c r="K60" s="75"/>
+      <c r="B60" s="78"/>
+      <c r="C60" s="78"/>
+      <c r="D60" s="78"/>
+      <c r="E60" s="78"/>
+      <c r="F60" s="78"/>
+      <c r="G60" s="78"/>
+      <c r="H60" s="78"/>
+      <c r="I60" s="78"/>
+      <c r="J60" s="78"/>
+      <c r="K60" s="78"/>
       <c r="L60" s="8"/>
     </row>
     <row r="61" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="76"/>
-      <c r="B61" s="77"/>
-      <c r="C61" s="77"/>
-      <c r="D61" s="77"/>
-      <c r="E61" s="77"/>
-      <c r="F61" s="77"/>
-      <c r="G61" s="77"/>
-      <c r="H61" s="77"/>
-      <c r="I61" s="77"/>
-      <c r="J61" s="77"/>
-      <c r="K61" s="78"/>
+      <c r="A61" s="79"/>
+      <c r="B61" s="80"/>
+      <c r="C61" s="80"/>
+      <c r="D61" s="80"/>
+      <c r="E61" s="80"/>
+      <c r="F61" s="80"/>
+      <c r="G61" s="80"/>
+      <c r="H61" s="80"/>
+      <c r="I61" s="80"/>
+      <c r="J61" s="80"/>
+      <c r="K61" s="81"/>
       <c r="L61" s="8"/>
     </row>
     <row r="62" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="76"/>
-      <c r="B62" s="77"/>
-      <c r="C62" s="77"/>
-      <c r="D62" s="77"/>
-      <c r="E62" s="77"/>
-      <c r="F62" s="77"/>
-      <c r="G62" s="77"/>
-      <c r="H62" s="77"/>
-      <c r="I62" s="77"/>
-      <c r="J62" s="77"/>
-      <c r="K62" s="76"/>
-      <c r="L62" s="76"/>
+      <c r="A62" s="79"/>
+      <c r="B62" s="80"/>
+      <c r="C62" s="80"/>
+      <c r="D62" s="80"/>
+      <c r="E62" s="80"/>
+      <c r="F62" s="80"/>
+      <c r="G62" s="80"/>
+      <c r="H62" s="80"/>
+      <c r="I62" s="80"/>
+      <c r="J62" s="80"/>
+      <c r="K62" s="79"/>
+      <c r="L62" s="79"/>
     </row>
     <row r="63" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="76"/>
-      <c r="B63" s="77"/>
-      <c r="C63" s="77"/>
-      <c r="D63" s="77"/>
-      <c r="E63" s="77"/>
-      <c r="F63" s="77"/>
-      <c r="G63" s="77"/>
-      <c r="H63" s="77"/>
-      <c r="I63" s="77"/>
-      <c r="J63" s="77"/>
-      <c r="K63" s="76"/>
-      <c r="L63" s="66"/>
+      <c r="A63" s="79"/>
+      <c r="B63" s="80"/>
+      <c r="C63" s="80"/>
+      <c r="D63" s="80"/>
+      <c r="E63" s="80"/>
+      <c r="F63" s="80"/>
+      <c r="G63" s="80"/>
+      <c r="H63" s="80"/>
+      <c r="I63" s="80"/>
+      <c r="J63" s="80"/>
+      <c r="K63" s="79"/>
+      <c r="L63" s="69"/>
     </row>
     <row r="64" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="79"/>
-      <c r="B64" s="80"/>
-      <c r="C64" s="81"/>
-      <c r="D64" s="81"/>
-      <c r="E64" s="81"/>
-      <c r="F64" s="80"/>
-      <c r="G64" s="80"/>
-      <c r="H64" s="80"/>
-      <c r="I64" s="81"/>
-      <c r="J64" s="81"/>
-      <c r="K64" s="81"/>
+      <c r="A64" s="82"/>
+      <c r="B64" s="83"/>
+      <c r="C64" s="84"/>
+      <c r="D64" s="84"/>
+      <c r="E64" s="84"/>
+      <c r="F64" s="83"/>
+      <c r="G64" s="83"/>
+      <c r="H64" s="83"/>
+      <c r="I64" s="84"/>
+      <c r="J64" s="84"/>
+      <c r="K64" s="84"/>
       <c r="L64" s="8"/>
     </row>
     <row r="65" ht="30" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="79"/>
-      <c r="B65" s="80"/>
-      <c r="C65" s="81"/>
-      <c r="D65" s="81"/>
-      <c r="E65" s="81"/>
-      <c r="F65" s="80"/>
+      <c r="A65" s="82"/>
+      <c r="B65" s="83"/>
+      <c r="C65" s="84"/>
+      <c r="D65" s="84"/>
+      <c r="E65" s="84"/>
+      <c r="F65" s="83"/>
       <c r="G65" s="8"/>
-      <c r="H65" s="80"/>
-      <c r="I65" s="80"/>
+      <c r="H65" s="83"/>
+      <c r="I65" s="83"/>
       <c r="J65" s="8"/>
       <c r="K65" s="8"/>
       <c r="L65" s="8"/>
     </row>
     <row r="66" ht="30" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="82"/>
-      <c r="B66" s="83"/>
-      <c r="C66" s="84"/>
-      <c r="D66" s="84"/>
-      <c r="E66" s="84"/>
-      <c r="F66" s="83"/>
-      <c r="G66" s="85"/>
-      <c r="H66" s="83"/>
-      <c r="I66" s="83"/>
-      <c r="J66" s="85"/>
-      <c r="K66" s="85"/>
+      <c r="A66" s="85"/>
+      <c r="B66" s="86"/>
+      <c r="C66" s="87"/>
+      <c r="D66" s="87"/>
+      <c r="E66" s="87"/>
+      <c r="F66" s="86"/>
+      <c r="G66" s="88"/>
+      <c r="H66" s="86"/>
+      <c r="I66" s="86"/>
+      <c r="J66" s="88"/>
+      <c r="K66" s="88"/>
       <c r="L66" s="8"/>
     </row>
     <row r="67" ht="19.5" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="86" t="s">
+      <c r="A67" s="89" t="s">
         <v>81</v>
       </c>
-      <c r="B67" s="86"/>
-      <c r="C67" s="86"/>
-      <c r="D67" s="87"/>
-      <c r="E67" s="87"/>
-      <c r="F67" s="88"/>
-      <c r="G67" s="89"/>
-      <c r="H67" s="90" t="s">
+      <c r="B67" s="89"/>
+      <c r="C67" s="89"/>
+      <c r="D67" s="90"/>
+      <c r="E67" s="90"/>
+      <c r="F67" s="91"/>
+      <c r="G67" s="92"/>
+      <c r="H67" s="93" t="s">
         <v>82</v>
       </c>
-      <c r="I67" s="90"/>
-      <c r="J67" s="90"/>
-      <c r="K67" s="90"/>
-      <c r="L67" s="91"/>
+      <c r="I67" s="93"/>
+      <c r="J67" s="93"/>
+      <c r="K67" s="93"/>
+      <c r="L67" s="94"/>
     </row>
     <row r="68" ht="20.1" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="88" t="s">
+      <c r="A68" s="91" t="s">
         <v>83</v>
       </c>
-      <c r="B68" s="88"/>
-      <c r="C68" s="88"/>
-      <c r="D68" s="88"/>
-      <c r="E68" s="88"/>
-      <c r="F68" s="88"/>
-      <c r="G68" s="89"/>
-      <c r="H68" s="88" t="s">
+      <c r="B68" s="91"/>
+      <c r="C68" s="91"/>
+      <c r="D68" s="91"/>
+      <c r="E68" s="91"/>
+      <c r="F68" s="91"/>
+      <c r="G68" s="92"/>
+      <c r="H68" s="91" t="s">
         <v>84</v>
       </c>
-      <c r="I68" s="88"/>
-      <c r="J68" s="88"/>
-      <c r="K68" s="88"/>
+      <c r="I68" s="91"/>
+      <c r="J68" s="91"/>
+      <c r="K68" s="91"/>
       <c r="L68" s="12"/>
     </row>
     <row r="69" ht="30" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="88"/>
-      <c r="B69" s="88"/>
-      <c r="C69" s="88"/>
-      <c r="D69" s="88"/>
-      <c r="E69" s="88"/>
-      <c r="F69" s="88"/>
-      <c r="G69" s="89"/>
-      <c r="H69" s="88"/>
-      <c r="I69" s="88"/>
-      <c r="J69" s="88"/>
-      <c r="K69" s="88"/>
+      <c r="A69" s="91"/>
+      <c r="B69" s="91"/>
+      <c r="C69" s="91"/>
+      <c r="D69" s="91"/>
+      <c r="E69" s="91"/>
+      <c r="F69" s="91"/>
+      <c r="G69" s="92"/>
+      <c r="H69" s="91"/>
+      <c r="I69" s="91"/>
+      <c r="J69" s="91"/>
+      <c r="K69" s="91"/>
       <c r="L69" s="12"/>
     </row>
     <row r="70" ht="30" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="88"/>
-      <c r="B70" s="88"/>
-      <c r="C70" s="88"/>
-      <c r="D70" s="88"/>
-      <c r="E70" s="88"/>
-      <c r="F70" s="88"/>
-      <c r="G70" s="89"/>
-      <c r="H70" s="88"/>
-      <c r="I70" s="88"/>
-      <c r="J70" s="88"/>
-      <c r="K70" s="88"/>
+      <c r="A70" s="91"/>
+      <c r="B70" s="91"/>
+      <c r="C70" s="91"/>
+      <c r="D70" s="91"/>
+      <c r="E70" s="91"/>
+      <c r="F70" s="91"/>
+      <c r="G70" s="92"/>
+      <c r="H70" s="91"/>
+      <c r="I70" s="91"/>
+      <c r="J70" s="91"/>
+      <c r="K70" s="91"/>
       <c r="L70" s="12"/>
     </row>
     <row r="71" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="88"/>
-      <c r="B71" s="88"/>
-      <c r="C71" s="88"/>
-      <c r="D71" s="88"/>
-      <c r="E71" s="88"/>
-      <c r="F71" s="88"/>
-      <c r="G71" s="89"/>
-      <c r="H71" s="88"/>
-      <c r="I71" s="88"/>
-      <c r="J71" s="88"/>
-      <c r="K71" s="88"/>
+      <c r="A71" s="91"/>
+      <c r="B71" s="91"/>
+      <c r="C71" s="91"/>
+      <c r="D71" s="91"/>
+      <c r="E71" s="91"/>
+      <c r="F71" s="91"/>
+      <c r="G71" s="92"/>
+      <c r="H71" s="91"/>
+      <c r="I71" s="91"/>
+      <c r="J71" s="91"/>
+      <c r="K71" s="91"/>
       <c r="L71" s="12"/>
     </row>
     <row r="72" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="88"/>
-      <c r="B72" s="88"/>
-      <c r="C72" s="89"/>
-      <c r="D72" s="89"/>
-      <c r="E72" s="89"/>
-      <c r="F72" s="88"/>
-      <c r="G72" s="89"/>
-      <c r="H72" s="88"/>
-      <c r="I72" s="88"/>
-      <c r="J72" s="89"/>
-      <c r="K72" s="89"/>
+      <c r="A72" s="91"/>
+      <c r="B72" s="91"/>
+      <c r="C72" s="92"/>
+      <c r="D72" s="92"/>
+      <c r="E72" s="92"/>
+      <c r="F72" s="91"/>
+      <c r="G72" s="92"/>
+      <c r="H72" s="91"/>
+      <c r="I72" s="91"/>
+      <c r="J72" s="92"/>
+      <c r="K72" s="92"/>
       <c r="L72" s="12"/>
     </row>
     <row r="73" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="92"/>
-      <c r="B73" s="92"/>
-      <c r="C73" s="92"/>
-      <c r="D73" s="93"/>
-      <c r="E73" s="93"/>
-      <c r="F73" s="94"/>
-      <c r="G73" s="95"/>
-      <c r="H73" s="92"/>
-      <c r="I73" s="92"/>
-      <c r="J73" s="92"/>
-      <c r="K73" s="92"/>
-      <c r="L73" s="96"/>
+      <c r="A73" s="95"/>
+      <c r="B73" s="95"/>
+      <c r="C73" s="95"/>
+      <c r="D73" s="96"/>
+      <c r="E73" s="96"/>
+      <c r="F73" s="97"/>
+      <c r="G73" s="98"/>
+      <c r="H73" s="95"/>
+      <c r="I73" s="95"/>
+      <c r="J73" s="95"/>
+      <c r="K73" s="95"/>
+      <c r="L73" s="99"/>
     </row>
     <row r="74" ht="18.75" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="97" t="s">
+      <c r="A74" s="100" t="s">
         <v>85</v>
       </c>
-      <c r="B74" s="97"/>
-      <c r="C74" s="97"/>
-      <c r="D74" s="93"/>
-      <c r="E74" s="93"/>
-      <c r="F74" s="94"/>
-      <c r="G74" s="95"/>
-      <c r="H74" s="88" t="s">
+      <c r="B74" s="100"/>
+      <c r="C74" s="100"/>
+      <c r="D74" s="96"/>
+      <c r="E74" s="96"/>
+      <c r="F74" s="97"/>
+      <c r="G74" s="98"/>
+      <c r="H74" s="91" t="s">
         <v>86</v>
       </c>
-      <c r="I74" s="88"/>
-      <c r="J74" s="88"/>
-      <c r="K74" s="88"/>
+      <c r="I74" s="91"/>
+      <c r="J74" s="91"/>
+      <c r="K74" s="91"/>
       <c r="L74" s="8"/>
     </row>
     <row r="75" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="88" t="s">
+      <c r="A75" s="91" t="s">
         <v>87</v>
       </c>
-      <c r="B75" s="88"/>
-      <c r="C75" s="88"/>
-      <c r="D75" s="88"/>
-      <c r="E75" s="88"/>
-      <c r="F75" s="87"/>
-      <c r="G75" s="93"/>
-      <c r="H75" s="87" t="s">
+      <c r="B75" s="91"/>
+      <c r="C75" s="91"/>
+      <c r="D75" s="91"/>
+      <c r="E75" s="91"/>
+      <c r="F75" s="90"/>
+      <c r="G75" s="96"/>
+      <c r="H75" s="90" t="s">
         <v>88</v>
       </c>
-      <c r="I75" s="87"/>
-      <c r="J75" s="87"/>
-      <c r="K75" s="87"/>
-      <c r="L75" s="96"/>
+      <c r="I75" s="90"/>
+      <c r="J75" s="90"/>
+      <c r="K75" s="90"/>
+      <c r="L75" s="99"/>
     </row>
     <row r="76" ht="20.25" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="98"/>
-      <c r="B76" s="98"/>
-      <c r="C76" s="98"/>
-      <c r="D76" s="83"/>
-      <c r="E76" s="83"/>
-      <c r="F76" s="99"/>
-      <c r="G76" s="100"/>
-      <c r="H76" s="101"/>
-      <c r="I76" s="101"/>
-      <c r="J76" s="101"/>
-      <c r="K76" s="102"/>
-      <c r="L76" s="103"/>
+      <c r="A76" s="101"/>
+      <c r="B76" s="101"/>
+      <c r="C76" s="101"/>
+      <c r="D76" s="86"/>
+      <c r="E76" s="86"/>
+      <c r="F76" s="102"/>
+      <c r="G76" s="103"/>
+      <c r="H76" s="104"/>
+      <c r="I76" s="104"/>
+      <c r="J76" s="104"/>
+      <c r="K76" s="105"/>
+      <c r="L76" s="106"/>
     </row>
     <row r="77" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="104"/>
-      <c r="B77" s="104"/>
-      <c r="C77" s="104"/>
-      <c r="D77" s="105"/>
-      <c r="E77" s="105"/>
+      <c r="A77" s="107"/>
+      <c r="B77" s="107"/>
+      <c r="C77" s="107"/>
+      <c r="D77" s="108"/>
+      <c r="E77" s="108"/>
       <c r="F77" s="2"/>
-      <c r="G77" s="106"/>
-      <c r="H77" s="107" t="s">
+      <c r="G77" s="109"/>
+      <c r="H77" s="110" t="s">
         <v>89</v>
       </c>
-      <c r="I77" s="107"/>
-      <c r="J77" s="107"/>
-      <c r="K77" s="107"/>
+      <c r="I77" s="110"/>
+      <c r="J77" s="110"/>
+      <c r="K77" s="110"/>
       <c r="L77" s="2"/>
     </row>
     <row r="78" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="104"/>
-      <c r="B78" s="104"/>
-      <c r="C78" s="104"/>
+      <c r="A78" s="107"/>
+      <c r="B78" s="107"/>
+      <c r="C78" s="107"/>
       <c r="D78" s="2"/>
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
-      <c r="G78" s="106"/>
-      <c r="H78" s="107"/>
-      <c r="I78" s="107"/>
-      <c r="J78" s="107"/>
-      <c r="K78" s="107"/>
+      <c r="G78" s="109"/>
+      <c r="H78" s="110"/>
+      <c r="I78" s="110"/>
+      <c r="J78" s="110"/>
+      <c r="K78" s="110"/>
       <c r="L78" s="2"/>
     </row>
     <row r="79" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="104"/>
-      <c r="B79" s="104"/>
-      <c r="C79" s="104"/>
+      <c r="A79" s="107"/>
+      <c r="B79" s="107"/>
+      <c r="C79" s="107"/>
       <c r="D79" s="2"/>
       <c r="E79" s="2"/>
       <c r="F79" s="2"/>
-      <c r="G79" s="106"/>
-      <c r="H79" s="107"/>
-      <c r="I79" s="107"/>
-      <c r="J79" s="107"/>
-      <c r="K79" s="107"/>
+      <c r="G79" s="109"/>
+      <c r="H79" s="110"/>
+      <c r="I79" s="110"/>
+      <c r="J79" s="110"/>
+      <c r="K79" s="110"/>
       <c r="L79" s="2"/>
     </row>
     <row r="80" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="104"/>
-      <c r="B80" s="104"/>
-      <c r="C80" s="104"/>
+      <c r="A80" s="107"/>
+      <c r="B80" s="107"/>
+      <c r="C80" s="107"/>
       <c r="D80" s="2"/>
       <c r="E80" s="2"/>
       <c r="F80" s="2"/>
-      <c r="G80" s="106"/>
-      <c r="H80" s="107"/>
-      <c r="I80" s="107"/>
-      <c r="J80" s="107"/>
-      <c r="K80" s="107"/>
+      <c r="G80" s="109"/>
+      <c r="H80" s="110"/>
+      <c r="I80" s="110"/>
+      <c r="J80" s="110"/>
+      <c r="K80" s="110"/>
       <c r="L80" s="2"/>
     </row>
     <row r="81" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="104"/>
-      <c r="B81" s="104"/>
-      <c r="C81" s="104"/>
+      <c r="A81" s="107"/>
+      <c r="B81" s="107"/>
+      <c r="C81" s="107"/>
       <c r="D81" s="2"/>
       <c r="E81" s="2"/>
       <c r="F81" s="2"/>
-      <c r="G81" s="106"/>
-      <c r="H81" s="107"/>
-      <c r="I81" s="107"/>
-      <c r="J81" s="107"/>
-      <c r="K81" s="107"/>
+      <c r="G81" s="109"/>
+      <c r="H81" s="110"/>
+      <c r="I81" s="110"/>
+      <c r="J81" s="110"/>
+      <c r="K81" s="110"/>
       <c r="L81" s="2"/>
     </row>
     <row r="82" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="104"/>
-      <c r="B82" s="104"/>
-      <c r="C82" s="104"/>
+      <c r="A82" s="107"/>
+      <c r="B82" s="107"/>
+      <c r="C82" s="107"/>
       <c r="D82" s="2"/>
       <c r="E82" s="2"/>
       <c r="F82" s="2"/>
-      <c r="G82" s="106"/>
-      <c r="H82" s="107"/>
-      <c r="I82" s="107"/>
-      <c r="J82" s="107"/>
-      <c r="K82" s="107"/>
+      <c r="G82" s="109"/>
+      <c r="H82" s="110"/>
+      <c r="I82" s="110"/>
+      <c r="J82" s="110"/>
+      <c r="K82" s="110"/>
       <c r="L82" s="2"/>
     </row>
     <row r="83" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="104"/>
-      <c r="B83" s="104"/>
-      <c r="C83" s="104"/>
+      <c r="A83" s="107"/>
+      <c r="B83" s="107"/>
+      <c r="C83" s="107"/>
       <c r="D83" s="2"/>
       <c r="E83" s="2"/>
       <c r="F83" s="2"/>
-      <c r="G83" s="106"/>
-      <c r="H83" s="107"/>
-      <c r="I83" s="107"/>
-      <c r="J83" s="107"/>
-      <c r="K83" s="107"/>
+      <c r="G83" s="109"/>
+      <c r="H83" s="110"/>
+      <c r="I83" s="110"/>
+      <c r="J83" s="110"/>
+      <c r="K83" s="110"/>
       <c r="L83" s="2"/>
     </row>
     <row r="84" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="104"/>
-      <c r="B84" s="104"/>
-      <c r="C84" s="104"/>
+      <c r="A84" s="107"/>
+      <c r="B84" s="107"/>
+      <c r="C84" s="107"/>
       <c r="D84" s="2"/>
       <c r="E84" s="2"/>
       <c r="F84" s="2"/>
-      <c r="G84" s="106"/>
-      <c r="H84" s="107"/>
-      <c r="I84" s="107"/>
-      <c r="J84" s="107"/>
-      <c r="K84" s="107"/>
+      <c r="G84" s="109"/>
+      <c r="H84" s="110"/>
+      <c r="I84" s="110"/>
+      <c r="J84" s="110"/>
+      <c r="K84" s="110"/>
       <c r="L84" s="2"/>
     </row>
     <row r="85" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="104"/>
-      <c r="B85" s="104"/>
-      <c r="C85" s="104"/>
+      <c r="A85" s="107"/>
+      <c r="B85" s="107"/>
+      <c r="C85" s="107"/>
       <c r="D85" s="2"/>
       <c r="E85" s="2"/>
       <c r="F85" s="2"/>
-      <c r="G85" s="106"/>
-      <c r="H85" s="107"/>
-      <c r="I85" s="107"/>
-      <c r="J85" s="107"/>
-      <c r="K85" s="107"/>
+      <c r="G85" s="109"/>
+      <c r="H85" s="110"/>
+      <c r="I85" s="110"/>
+      <c r="J85" s="110"/>
+      <c r="K85" s="110"/>
       <c r="L85" s="2"/>
     </row>
     <row r="86" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="104"/>
-      <c r="B86" s="104"/>
-      <c r="C86" s="104"/>
+      <c r="A86" s="107"/>
+      <c r="B86" s="107"/>
+      <c r="C86" s="107"/>
       <c r="D86" s="2"/>
       <c r="E86" s="2"/>
       <c r="F86" s="2"/>
-      <c r="G86" s="106"/>
-      <c r="H86" s="107"/>
-      <c r="I86" s="107"/>
-      <c r="J86" s="107"/>
-      <c r="K86" s="107"/>
+      <c r="G86" s="109"/>
+      <c r="H86" s="110"/>
+      <c r="I86" s="110"/>
+      <c r="J86" s="110"/>
+      <c r="K86" s="110"/>
       <c r="L86" s="2"/>
     </row>
     <row r="87" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="104"/>
-      <c r="B87" s="104"/>
-      <c r="C87" s="104"/>
+      <c r="A87" s="107"/>
+      <c r="B87" s="107"/>
+      <c r="C87" s="107"/>
       <c r="D87" s="2"/>
       <c r="E87" s="2"/>
       <c r="F87" s="2"/>
-      <c r="G87" s="106"/>
-      <c r="H87" s="107"/>
-      <c r="I87" s="107"/>
-      <c r="J87" s="107"/>
-      <c r="K87" s="107"/>
+      <c r="G87" s="109"/>
+      <c r="H87" s="110"/>
+      <c r="I87" s="110"/>
+      <c r="J87" s="110"/>
+      <c r="K87" s="110"/>
       <c r="L87" s="2"/>
     </row>
     <row r="88" ht="30" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A88" s="104"/>
-      <c r="B88" s="104"/>
-      <c r="C88" s="104"/>
+      <c r="A88" s="107"/>
+      <c r="B88" s="107"/>
+      <c r="C88" s="107"/>
       <c r="D88" s="2"/>
       <c r="E88" s="2"/>
       <c r="F88" s="2"/>
-      <c r="G88" s="106"/>
-      <c r="H88" s="107"/>
-      <c r="I88" s="107"/>
-      <c r="J88" s="107"/>
-      <c r="K88" s="107"/>
+      <c r="G88" s="109"/>
+      <c r="H88" s="110"/>
+      <c r="I88" s="110"/>
+      <c r="J88" s="110"/>
+      <c r="K88" s="110"/>
       <c r="L88" s="2"/>
     </row>
     <row r="89" ht="30" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A89" s="104"/>
-      <c r="B89" s="104"/>
-      <c r="C89" s="104"/>
+      <c r="A89" s="107"/>
+      <c r="B89" s="107"/>
+      <c r="C89" s="107"/>
       <c r="D89" s="2"/>
       <c r="E89" s="2"/>
       <c r="F89" s="2"/>
       <c r="G89" s="2"/>
-      <c r="H89" s="107"/>
-      <c r="I89" s="107"/>
-      <c r="J89" s="107"/>
-      <c r="K89" s="107"/>
+      <c r="H89" s="110"/>
+      <c r="I89" s="110"/>
+      <c r="J89" s="110"/>
+      <c r="K89" s="110"/>
       <c r="L89" s="2"/>
     </row>
     <row r="90" spans="13:17" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
fix(requisiciones): no perder el borde grueso de los demás biológicos al agregar lotes
ExcelJS comparte el objeto de estilo entre celdas con el mismo formato: cambiar solo el
borde de una celda cambiaba todas las del grupo (las columnas de lote y caducidad perdían
el borde grueso en todos los biológicos). Ahora se reasigna el estilo completo por celda,
también en el script que genera la plantilla.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/requisiciones_plantilla.xlsx
+++ b/requisiciones_plantilla.xlsx
@@ -452,7 +452,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="30">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -783,6 +783,30 @@
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -831,7 +855,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -1027,10 +1051,22 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="12" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1118,7 +1154,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1130,7 +1166,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -1153,11 +1189,11 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1166,17 +1202,17 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1188,8 +1224,12 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -2668,519 +2708,519 @@
       <c r="L54" s="1"/>
     </row>
     <row r="55" ht="26.25" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="56"/>
-      <c r="B55" s="57"/>
-      <c r="C55" s="58"/>
-      <c r="D55" s="59"/>
-      <c r="E55" s="60"/>
-      <c r="F55" s="61"/>
+      <c r="A55" s="64"/>
+      <c r="B55" s="65"/>
+      <c r="C55" s="66"/>
+      <c r="D55" s="38"/>
+      <c r="E55" s="39"/>
+      <c r="F55" s="40"/>
       <c r="G55" s="47"/>
       <c r="H55" s="47"/>
       <c r="I55" s="48"/>
       <c r="J55" s="49"/>
-      <c r="K55" s="63"/>
+      <c r="K55" s="67"/>
       <c r="L55" s="1"/>
     </row>
     <row r="56" ht="25.5" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="64"/>
-      <c r="B56" s="65" t="s">
+      <c r="A56" s="68"/>
+      <c r="B56" s="69" t="s">
         <v>77</v>
       </c>
-      <c r="C56" s="65"/>
-      <c r="D56" s="65"/>
-      <c r="E56" s="65"/>
-      <c r="F56" s="65"/>
-      <c r="G56" s="65"/>
-      <c r="H56" s="65"/>
-      <c r="I56" s="65"/>
-      <c r="J56" s="65"/>
-      <c r="K56" s="66"/>
+      <c r="C56" s="69"/>
+      <c r="D56" s="69"/>
+      <c r="E56" s="69"/>
+      <c r="F56" s="69"/>
+      <c r="G56" s="69"/>
+      <c r="H56" s="69"/>
+      <c r="I56" s="69"/>
+      <c r="J56" s="69"/>
+      <c r="K56" s="70"/>
       <c r="L56" s="55"/>
     </row>
     <row r="57" ht="25.5" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="67"/>
-      <c r="B57" s="68"/>
-      <c r="C57" s="69"/>
-      <c r="D57" s="70"/>
-      <c r="E57" s="70"/>
-      <c r="F57" s="70"/>
-      <c r="G57" s="71"/>
-      <c r="H57" s="71"/>
-      <c r="I57" s="72"/>
-      <c r="J57" s="73"/>
-      <c r="K57" s="74"/>
+      <c r="A57" s="71"/>
+      <c r="B57" s="72"/>
+      <c r="C57" s="73"/>
+      <c r="D57" s="74"/>
+      <c r="E57" s="74"/>
+      <c r="F57" s="74"/>
+      <c r="G57" s="75"/>
+      <c r="H57" s="75"/>
+      <c r="I57" s="76"/>
+      <c r="J57" s="77"/>
+      <c r="K57" s="78"/>
       <c r="L57" s="8"/>
     </row>
     <row r="58" ht="25.5" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="67"/>
+      <c r="A58" s="71"/>
       <c r="B58" s="8"/>
-      <c r="C58" s="75" t="s">
+      <c r="C58" s="79" t="s">
         <v>78</v>
       </c>
-      <c r="D58" s="76"/>
-      <c r="E58" s="72"/>
-      <c r="F58" s="70"/>
-      <c r="G58" s="75" t="s">
+      <c r="D58" s="80"/>
+      <c r="E58" s="76"/>
+      <c r="F58" s="74"/>
+      <c r="G58" s="79" t="s">
         <v>79</v>
       </c>
-      <c r="H58" s="75"/>
-      <c r="I58" s="77"/>
-      <c r="J58" s="73"/>
-      <c r="K58" s="74"/>
+      <c r="H58" s="79"/>
+      <c r="I58" s="81"/>
+      <c r="J58" s="77"/>
+      <c r="K58" s="78"/>
       <c r="L58" s="8"/>
     </row>
     <row r="59" ht="25.5" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="67"/>
-      <c r="B59" s="68"/>
-      <c r="C59" s="69"/>
-      <c r="D59" s="70"/>
-      <c r="E59" s="70"/>
-      <c r="F59" s="70"/>
-      <c r="G59" s="71"/>
-      <c r="H59" s="71"/>
-      <c r="I59" s="72"/>
-      <c r="J59" s="73"/>
-      <c r="K59" s="74"/>
+      <c r="A59" s="71"/>
+      <c r="B59" s="72"/>
+      <c r="C59" s="73"/>
+      <c r="D59" s="74"/>
+      <c r="E59" s="74"/>
+      <c r="F59" s="74"/>
+      <c r="G59" s="75"/>
+      <c r="H59" s="75"/>
+      <c r="I59" s="76"/>
+      <c r="J59" s="77"/>
+      <c r="K59" s="78"/>
       <c r="L59" s="8"/>
     </row>
     <row r="60" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="78" t="s">
+      <c r="A60" s="82" t="s">
         <v>80</v>
       </c>
-      <c r="B60" s="78"/>
-      <c r="C60" s="78"/>
-      <c r="D60" s="78"/>
-      <c r="E60" s="78"/>
-      <c r="F60" s="78"/>
-      <c r="G60" s="78"/>
-      <c r="H60" s="78"/>
-      <c r="I60" s="78"/>
-      <c r="J60" s="78"/>
-      <c r="K60" s="78"/>
+      <c r="B60" s="82"/>
+      <c r="C60" s="82"/>
+      <c r="D60" s="82"/>
+      <c r="E60" s="82"/>
+      <c r="F60" s="82"/>
+      <c r="G60" s="82"/>
+      <c r="H60" s="82"/>
+      <c r="I60" s="82"/>
+      <c r="J60" s="82"/>
+      <c r="K60" s="82"/>
       <c r="L60" s="8"/>
     </row>
     <row r="61" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="79"/>
-      <c r="B61" s="80"/>
-      <c r="C61" s="80"/>
-      <c r="D61" s="80"/>
-      <c r="E61" s="80"/>
-      <c r="F61" s="80"/>
-      <c r="G61" s="80"/>
-      <c r="H61" s="80"/>
-      <c r="I61" s="80"/>
-      <c r="J61" s="80"/>
-      <c r="K61" s="81"/>
+      <c r="A61" s="83"/>
+      <c r="B61" s="84"/>
+      <c r="C61" s="84"/>
+      <c r="D61" s="84"/>
+      <c r="E61" s="84"/>
+      <c r="F61" s="84"/>
+      <c r="G61" s="84"/>
+      <c r="H61" s="84"/>
+      <c r="I61" s="84"/>
+      <c r="J61" s="84"/>
+      <c r="K61" s="85"/>
       <c r="L61" s="8"/>
     </row>
     <row r="62" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="79"/>
-      <c r="B62" s="80"/>
-      <c r="C62" s="80"/>
-      <c r="D62" s="80"/>
-      <c r="E62" s="80"/>
-      <c r="F62" s="80"/>
-      <c r="G62" s="80"/>
-      <c r="H62" s="80"/>
-      <c r="I62" s="80"/>
-      <c r="J62" s="80"/>
-      <c r="K62" s="79"/>
-      <c r="L62" s="79"/>
+      <c r="A62" s="83"/>
+      <c r="B62" s="84"/>
+      <c r="C62" s="84"/>
+      <c r="D62" s="84"/>
+      <c r="E62" s="84"/>
+      <c r="F62" s="84"/>
+      <c r="G62" s="84"/>
+      <c r="H62" s="84"/>
+      <c r="I62" s="84"/>
+      <c r="J62" s="84"/>
+      <c r="K62" s="83"/>
+      <c r="L62" s="83"/>
     </row>
     <row r="63" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="79"/>
-      <c r="B63" s="80"/>
-      <c r="C63" s="80"/>
-      <c r="D63" s="80"/>
-      <c r="E63" s="80"/>
-      <c r="F63" s="80"/>
-      <c r="G63" s="80"/>
-      <c r="H63" s="80"/>
-      <c r="I63" s="80"/>
-      <c r="J63" s="80"/>
-      <c r="K63" s="79"/>
-      <c r="L63" s="69"/>
+      <c r="A63" s="83"/>
+      <c r="B63" s="84"/>
+      <c r="C63" s="84"/>
+      <c r="D63" s="84"/>
+      <c r="E63" s="84"/>
+      <c r="F63" s="84"/>
+      <c r="G63" s="84"/>
+      <c r="H63" s="84"/>
+      <c r="I63" s="84"/>
+      <c r="J63" s="84"/>
+      <c r="K63" s="83"/>
+      <c r="L63" s="73"/>
     </row>
     <row r="64" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="82"/>
-      <c r="B64" s="83"/>
-      <c r="C64" s="84"/>
-      <c r="D64" s="84"/>
-      <c r="E64" s="84"/>
-      <c r="F64" s="83"/>
-      <c r="G64" s="83"/>
-      <c r="H64" s="83"/>
-      <c r="I64" s="84"/>
-      <c r="J64" s="84"/>
-      <c r="K64" s="84"/>
+      <c r="A64" s="86"/>
+      <c r="B64" s="87"/>
+      <c r="C64" s="88"/>
+      <c r="D64" s="88"/>
+      <c r="E64" s="88"/>
+      <c r="F64" s="87"/>
+      <c r="G64" s="87"/>
+      <c r="H64" s="87"/>
+      <c r="I64" s="88"/>
+      <c r="J64" s="88"/>
+      <c r="K64" s="88"/>
       <c r="L64" s="8"/>
     </row>
     <row r="65" ht="30" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="82"/>
-      <c r="B65" s="83"/>
-      <c r="C65" s="84"/>
-      <c r="D65" s="84"/>
-      <c r="E65" s="84"/>
-      <c r="F65" s="83"/>
+      <c r="A65" s="86"/>
+      <c r="B65" s="87"/>
+      <c r="C65" s="88"/>
+      <c r="D65" s="88"/>
+      <c r="E65" s="88"/>
+      <c r="F65" s="87"/>
       <c r="G65" s="8"/>
-      <c r="H65" s="83"/>
-      <c r="I65" s="83"/>
+      <c r="H65" s="87"/>
+      <c r="I65" s="87"/>
       <c r="J65" s="8"/>
       <c r="K65" s="8"/>
       <c r="L65" s="8"/>
     </row>
     <row r="66" ht="30" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="85"/>
-      <c r="B66" s="86"/>
-      <c r="C66" s="87"/>
-      <c r="D66" s="87"/>
-      <c r="E66" s="87"/>
-      <c r="F66" s="86"/>
-      <c r="G66" s="88"/>
-      <c r="H66" s="86"/>
-      <c r="I66" s="86"/>
-      <c r="J66" s="88"/>
-      <c r="K66" s="88"/>
+      <c r="A66" s="89"/>
+      <c r="B66" s="90"/>
+      <c r="C66" s="91"/>
+      <c r="D66" s="91"/>
+      <c r="E66" s="91"/>
+      <c r="F66" s="90"/>
+      <c r="G66" s="92"/>
+      <c r="H66" s="90"/>
+      <c r="I66" s="90"/>
+      <c r="J66" s="92"/>
+      <c r="K66" s="92"/>
       <c r="L66" s="8"/>
     </row>
     <row r="67" ht="19.5" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="89" t="s">
+      <c r="A67" s="93" t="s">
         <v>81</v>
       </c>
-      <c r="B67" s="89"/>
-      <c r="C67" s="89"/>
-      <c r="D67" s="90"/>
-      <c r="E67" s="90"/>
-      <c r="F67" s="91"/>
-      <c r="G67" s="92"/>
-      <c r="H67" s="93" t="s">
+      <c r="B67" s="93"/>
+      <c r="C67" s="93"/>
+      <c r="D67" s="94"/>
+      <c r="E67" s="94"/>
+      <c r="F67" s="95"/>
+      <c r="G67" s="96"/>
+      <c r="H67" s="97" t="s">
         <v>82</v>
       </c>
-      <c r="I67" s="93"/>
-      <c r="J67" s="93"/>
-      <c r="K67" s="93"/>
-      <c r="L67" s="94"/>
+      <c r="I67" s="97"/>
+      <c r="J67" s="97"/>
+      <c r="K67" s="97"/>
+      <c r="L67" s="98"/>
     </row>
     <row r="68" ht="20.1" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="91" t="s">
+      <c r="A68" s="95" t="s">
         <v>83</v>
       </c>
-      <c r="B68" s="91"/>
-      <c r="C68" s="91"/>
-      <c r="D68" s="91"/>
-      <c r="E68" s="91"/>
-      <c r="F68" s="91"/>
-      <c r="G68" s="92"/>
-      <c r="H68" s="91" t="s">
+      <c r="B68" s="95"/>
+      <c r="C68" s="95"/>
+      <c r="D68" s="95"/>
+      <c r="E68" s="95"/>
+      <c r="F68" s="95"/>
+      <c r="G68" s="96"/>
+      <c r="H68" s="95" t="s">
         <v>84</v>
       </c>
-      <c r="I68" s="91"/>
-      <c r="J68" s="91"/>
-      <c r="K68" s="91"/>
+      <c r="I68" s="95"/>
+      <c r="J68" s="95"/>
+      <c r="K68" s="95"/>
       <c r="L68" s="12"/>
     </row>
     <row r="69" ht="30" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="91"/>
-      <c r="B69" s="91"/>
-      <c r="C69" s="91"/>
-      <c r="D69" s="91"/>
-      <c r="E69" s="91"/>
-      <c r="F69" s="91"/>
-      <c r="G69" s="92"/>
-      <c r="H69" s="91"/>
-      <c r="I69" s="91"/>
-      <c r="J69" s="91"/>
-      <c r="K69" s="91"/>
+      <c r="A69" s="95"/>
+      <c r="B69" s="95"/>
+      <c r="C69" s="95"/>
+      <c r="D69" s="95"/>
+      <c r="E69" s="95"/>
+      <c r="F69" s="95"/>
+      <c r="G69" s="96"/>
+      <c r="H69" s="95"/>
+      <c r="I69" s="95"/>
+      <c r="J69" s="95"/>
+      <c r="K69" s="95"/>
       <c r="L69" s="12"/>
     </row>
     <row r="70" ht="30" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="91"/>
-      <c r="B70" s="91"/>
-      <c r="C70" s="91"/>
-      <c r="D70" s="91"/>
-      <c r="E70" s="91"/>
-      <c r="F70" s="91"/>
-      <c r="G70" s="92"/>
-      <c r="H70" s="91"/>
-      <c r="I70" s="91"/>
-      <c r="J70" s="91"/>
-      <c r="K70" s="91"/>
+      <c r="A70" s="95"/>
+      <c r="B70" s="95"/>
+      <c r="C70" s="95"/>
+      <c r="D70" s="95"/>
+      <c r="E70" s="95"/>
+      <c r="F70" s="95"/>
+      <c r="G70" s="96"/>
+      <c r="H70" s="95"/>
+      <c r="I70" s="95"/>
+      <c r="J70" s="95"/>
+      <c r="K70" s="95"/>
       <c r="L70" s="12"/>
     </row>
     <row r="71" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="91"/>
-      <c r="B71" s="91"/>
-      <c r="C71" s="91"/>
-      <c r="D71" s="91"/>
-      <c r="E71" s="91"/>
-      <c r="F71" s="91"/>
-      <c r="G71" s="92"/>
-      <c r="H71" s="91"/>
-      <c r="I71" s="91"/>
-      <c r="J71" s="91"/>
-      <c r="K71" s="91"/>
+      <c r="A71" s="95"/>
+      <c r="B71" s="95"/>
+      <c r="C71" s="95"/>
+      <c r="D71" s="95"/>
+      <c r="E71" s="95"/>
+      <c r="F71" s="95"/>
+      <c r="G71" s="96"/>
+      <c r="H71" s="95"/>
+      <c r="I71" s="95"/>
+      <c r="J71" s="95"/>
+      <c r="K71" s="95"/>
       <c r="L71" s="12"/>
     </row>
     <row r="72" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="91"/>
-      <c r="B72" s="91"/>
-      <c r="C72" s="92"/>
-      <c r="D72" s="92"/>
-      <c r="E72" s="92"/>
-      <c r="F72" s="91"/>
-      <c r="G72" s="92"/>
-      <c r="H72" s="91"/>
-      <c r="I72" s="91"/>
-      <c r="J72" s="92"/>
-      <c r="K72" s="92"/>
+      <c r="A72" s="95"/>
+      <c r="B72" s="95"/>
+      <c r="C72" s="96"/>
+      <c r="D72" s="96"/>
+      <c r="E72" s="96"/>
+      <c r="F72" s="95"/>
+      <c r="G72" s="96"/>
+      <c r="H72" s="95"/>
+      <c r="I72" s="95"/>
+      <c r="J72" s="96"/>
+      <c r="K72" s="96"/>
       <c r="L72" s="12"/>
     </row>
     <row r="73" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="95"/>
-      <c r="B73" s="95"/>
-      <c r="C73" s="95"/>
-      <c r="D73" s="96"/>
-      <c r="E73" s="96"/>
-      <c r="F73" s="97"/>
-      <c r="G73" s="98"/>
-      <c r="H73" s="95"/>
-      <c r="I73" s="95"/>
-      <c r="J73" s="95"/>
-      <c r="K73" s="95"/>
-      <c r="L73" s="99"/>
+      <c r="A73" s="99"/>
+      <c r="B73" s="99"/>
+      <c r="C73" s="99"/>
+      <c r="D73" s="100"/>
+      <c r="E73" s="100"/>
+      <c r="F73" s="101"/>
+      <c r="G73" s="102"/>
+      <c r="H73" s="99"/>
+      <c r="I73" s="99"/>
+      <c r="J73" s="99"/>
+      <c r="K73" s="99"/>
+      <c r="L73" s="103"/>
     </row>
     <row r="74" ht="18.75" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="100" t="s">
+      <c r="A74" s="104" t="s">
         <v>85</v>
       </c>
-      <c r="B74" s="100"/>
-      <c r="C74" s="100"/>
-      <c r="D74" s="96"/>
-      <c r="E74" s="96"/>
-      <c r="F74" s="97"/>
-      <c r="G74" s="98"/>
-      <c r="H74" s="91" t="s">
+      <c r="B74" s="104"/>
+      <c r="C74" s="104"/>
+      <c r="D74" s="100"/>
+      <c r="E74" s="100"/>
+      <c r="F74" s="101"/>
+      <c r="G74" s="102"/>
+      <c r="H74" s="95" t="s">
         <v>86</v>
       </c>
-      <c r="I74" s="91"/>
-      <c r="J74" s="91"/>
-      <c r="K74" s="91"/>
+      <c r="I74" s="95"/>
+      <c r="J74" s="95"/>
+      <c r="K74" s="95"/>
       <c r="L74" s="8"/>
     </row>
     <row r="75" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="91" t="s">
+      <c r="A75" s="95" t="s">
         <v>87</v>
       </c>
-      <c r="B75" s="91"/>
-      <c r="C75" s="91"/>
-      <c r="D75" s="91"/>
-      <c r="E75" s="91"/>
-      <c r="F75" s="90"/>
-      <c r="G75" s="96"/>
-      <c r="H75" s="90" t="s">
+      <c r="B75" s="95"/>
+      <c r="C75" s="95"/>
+      <c r="D75" s="95"/>
+      <c r="E75" s="95"/>
+      <c r="F75" s="94"/>
+      <c r="G75" s="100"/>
+      <c r="H75" s="94" t="s">
         <v>88</v>
       </c>
-      <c r="I75" s="90"/>
-      <c r="J75" s="90"/>
-      <c r="K75" s="90"/>
-      <c r="L75" s="99"/>
+      <c r="I75" s="94"/>
+      <c r="J75" s="94"/>
+      <c r="K75" s="94"/>
+      <c r="L75" s="103"/>
     </row>
     <row r="76" ht="20.25" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="101"/>
-      <c r="B76" s="101"/>
-      <c r="C76" s="101"/>
-      <c r="D76" s="86"/>
-      <c r="E76" s="86"/>
-      <c r="F76" s="102"/>
-      <c r="G76" s="103"/>
-      <c r="H76" s="104"/>
-      <c r="I76" s="104"/>
-      <c r="J76" s="104"/>
-      <c r="K76" s="105"/>
-      <c r="L76" s="106"/>
+      <c r="A76" s="105"/>
+      <c r="B76" s="105"/>
+      <c r="C76" s="105"/>
+      <c r="D76" s="90"/>
+      <c r="E76" s="90"/>
+      <c r="F76" s="106"/>
+      <c r="G76" s="107"/>
+      <c r="H76" s="108"/>
+      <c r="I76" s="108"/>
+      <c r="J76" s="108"/>
+      <c r="K76" s="109"/>
+      <c r="L76" s="110"/>
     </row>
     <row r="77" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="107"/>
-      <c r="B77" s="107"/>
-      <c r="C77" s="107"/>
-      <c r="D77" s="108"/>
-      <c r="E77" s="108"/>
+      <c r="A77" s="111"/>
+      <c r="B77" s="111"/>
+      <c r="C77" s="111"/>
+      <c r="D77" s="112"/>
+      <c r="E77" s="112"/>
       <c r="F77" s="2"/>
-      <c r="G77" s="109"/>
-      <c r="H77" s="110" t="s">
+      <c r="G77" s="113"/>
+      <c r="H77" s="114" t="s">
         <v>89</v>
       </c>
-      <c r="I77" s="110"/>
-      <c r="J77" s="110"/>
-      <c r="K77" s="110"/>
+      <c r="I77" s="115"/>
+      <c r="J77" s="115"/>
+      <c r="K77" s="115"/>
       <c r="L77" s="2"/>
     </row>
     <row r="78" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="107"/>
-      <c r="B78" s="107"/>
-      <c r="C78" s="107"/>
+      <c r="A78" s="111"/>
+      <c r="B78" s="111"/>
+      <c r="C78" s="111"/>
       <c r="D78" s="2"/>
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
-      <c r="G78" s="109"/>
-      <c r="H78" s="110"/>
-      <c r="I78" s="110"/>
-      <c r="J78" s="110"/>
-      <c r="K78" s="110"/>
+      <c r="G78" s="113"/>
+      <c r="H78" s="115"/>
+      <c r="I78" s="115"/>
+      <c r="J78" s="115"/>
+      <c r="K78" s="115"/>
       <c r="L78" s="2"/>
     </row>
     <row r="79" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="107"/>
-      <c r="B79" s="107"/>
-      <c r="C79" s="107"/>
+      <c r="A79" s="111"/>
+      <c r="B79" s="111"/>
+      <c r="C79" s="111"/>
       <c r="D79" s="2"/>
       <c r="E79" s="2"/>
       <c r="F79" s="2"/>
-      <c r="G79" s="109"/>
-      <c r="H79" s="110"/>
-      <c r="I79" s="110"/>
-      <c r="J79" s="110"/>
-      <c r="K79" s="110"/>
+      <c r="G79" s="113"/>
+      <c r="H79" s="115"/>
+      <c r="I79" s="115"/>
+      <c r="J79" s="115"/>
+      <c r="K79" s="115"/>
       <c r="L79" s="2"/>
     </row>
     <row r="80" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="107"/>
-      <c r="B80" s="107"/>
-      <c r="C80" s="107"/>
+      <c r="A80" s="111"/>
+      <c r="B80" s="111"/>
+      <c r="C80" s="111"/>
       <c r="D80" s="2"/>
       <c r="E80" s="2"/>
       <c r="F80" s="2"/>
-      <c r="G80" s="109"/>
-      <c r="H80" s="110"/>
-      <c r="I80" s="110"/>
-      <c r="J80" s="110"/>
-      <c r="K80" s="110"/>
+      <c r="G80" s="113"/>
+      <c r="H80" s="115"/>
+      <c r="I80" s="115"/>
+      <c r="J80" s="115"/>
+      <c r="K80" s="115"/>
       <c r="L80" s="2"/>
     </row>
     <row r="81" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="107"/>
-      <c r="B81" s="107"/>
-      <c r="C81" s="107"/>
+      <c r="A81" s="111"/>
+      <c r="B81" s="111"/>
+      <c r="C81" s="111"/>
       <c r="D81" s="2"/>
       <c r="E81" s="2"/>
       <c r="F81" s="2"/>
-      <c r="G81" s="109"/>
-      <c r="H81" s="110"/>
-      <c r="I81" s="110"/>
-      <c r="J81" s="110"/>
-      <c r="K81" s="110"/>
+      <c r="G81" s="113"/>
+      <c r="H81" s="115"/>
+      <c r="I81" s="115"/>
+      <c r="J81" s="115"/>
+      <c r="K81" s="115"/>
       <c r="L81" s="2"/>
     </row>
     <row r="82" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="107"/>
-      <c r="B82" s="107"/>
-      <c r="C82" s="107"/>
+      <c r="A82" s="111"/>
+      <c r="B82" s="111"/>
+      <c r="C82" s="111"/>
       <c r="D82" s="2"/>
       <c r="E82" s="2"/>
       <c r="F82" s="2"/>
-      <c r="G82" s="109"/>
-      <c r="H82" s="110"/>
-      <c r="I82" s="110"/>
-      <c r="J82" s="110"/>
-      <c r="K82" s="110"/>
+      <c r="G82" s="113"/>
+      <c r="H82" s="115"/>
+      <c r="I82" s="115"/>
+      <c r="J82" s="115"/>
+      <c r="K82" s="115"/>
       <c r="L82" s="2"/>
     </row>
     <row r="83" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="107"/>
-      <c r="B83" s="107"/>
-      <c r="C83" s="107"/>
+      <c r="A83" s="111"/>
+      <c r="B83" s="111"/>
+      <c r="C83" s="111"/>
       <c r="D83" s="2"/>
       <c r="E83" s="2"/>
       <c r="F83" s="2"/>
-      <c r="G83" s="109"/>
-      <c r="H83" s="110"/>
-      <c r="I83" s="110"/>
-      <c r="J83" s="110"/>
-      <c r="K83" s="110"/>
+      <c r="G83" s="113"/>
+      <c r="H83" s="115"/>
+      <c r="I83" s="115"/>
+      <c r="J83" s="115"/>
+      <c r="K83" s="115"/>
       <c r="L83" s="2"/>
     </row>
     <row r="84" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="107"/>
-      <c r="B84" s="107"/>
-      <c r="C84" s="107"/>
+      <c r="A84" s="111"/>
+      <c r="B84" s="111"/>
+      <c r="C84" s="111"/>
       <c r="D84" s="2"/>
       <c r="E84" s="2"/>
       <c r="F84" s="2"/>
-      <c r="G84" s="109"/>
-      <c r="H84" s="110"/>
-      <c r="I84" s="110"/>
-      <c r="J84" s="110"/>
-      <c r="K84" s="110"/>
+      <c r="G84" s="113"/>
+      <c r="H84" s="115"/>
+      <c r="I84" s="115"/>
+      <c r="J84" s="115"/>
+      <c r="K84" s="115"/>
       <c r="L84" s="2"/>
     </row>
     <row r="85" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="107"/>
-      <c r="B85" s="107"/>
-      <c r="C85" s="107"/>
+      <c r="A85" s="111"/>
+      <c r="B85" s="111"/>
+      <c r="C85" s="111"/>
       <c r="D85" s="2"/>
       <c r="E85" s="2"/>
       <c r="F85" s="2"/>
-      <c r="G85" s="109"/>
-      <c r="H85" s="110"/>
-      <c r="I85" s="110"/>
-      <c r="J85" s="110"/>
-      <c r="K85" s="110"/>
+      <c r="G85" s="113"/>
+      <c r="H85" s="115"/>
+      <c r="I85" s="115"/>
+      <c r="J85" s="115"/>
+      <c r="K85" s="115"/>
       <c r="L85" s="2"/>
     </row>
     <row r="86" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="107"/>
-      <c r="B86" s="107"/>
-      <c r="C86" s="107"/>
+      <c r="A86" s="111"/>
+      <c r="B86" s="111"/>
+      <c r="C86" s="111"/>
       <c r="D86" s="2"/>
       <c r="E86" s="2"/>
       <c r="F86" s="2"/>
-      <c r="G86" s="109"/>
-      <c r="H86" s="110"/>
-      <c r="I86" s="110"/>
-      <c r="J86" s="110"/>
-      <c r="K86" s="110"/>
+      <c r="G86" s="113"/>
+      <c r="H86" s="115"/>
+      <c r="I86" s="115"/>
+      <c r="J86" s="115"/>
+      <c r="K86" s="115"/>
       <c r="L86" s="2"/>
     </row>
     <row r="87" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="107"/>
-      <c r="B87" s="107"/>
-      <c r="C87" s="107"/>
+      <c r="A87" s="111"/>
+      <c r="B87" s="111"/>
+      <c r="C87" s="111"/>
       <c r="D87" s="2"/>
       <c r="E87" s="2"/>
       <c r="F87" s="2"/>
-      <c r="G87" s="109"/>
-      <c r="H87" s="110"/>
-      <c r="I87" s="110"/>
-      <c r="J87" s="110"/>
-      <c r="K87" s="110"/>
+      <c r="G87" s="113"/>
+      <c r="H87" s="115"/>
+      <c r="I87" s="115"/>
+      <c r="J87" s="115"/>
+      <c r="K87" s="115"/>
       <c r="L87" s="2"/>
     </row>
     <row r="88" ht="30" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A88" s="107"/>
-      <c r="B88" s="107"/>
-      <c r="C88" s="107"/>
+      <c r="A88" s="111"/>
+      <c r="B88" s="111"/>
+      <c r="C88" s="111"/>
       <c r="D88" s="2"/>
       <c r="E88" s="2"/>
       <c r="F88" s="2"/>
-      <c r="G88" s="109"/>
-      <c r="H88" s="110"/>
-      <c r="I88" s="110"/>
-      <c r="J88" s="110"/>
-      <c r="K88" s="110"/>
+      <c r="G88" s="113"/>
+      <c r="H88" s="115"/>
+      <c r="I88" s="115"/>
+      <c r="J88" s="115"/>
+      <c r="K88" s="115"/>
       <c r="L88" s="2"/>
     </row>
     <row r="89" ht="30" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A89" s="107"/>
-      <c r="B89" s="107"/>
-      <c r="C89" s="107"/>
+      <c r="A89" s="111"/>
+      <c r="B89" s="111"/>
+      <c r="C89" s="111"/>
       <c r="D89" s="2"/>
       <c r="E89" s="2"/>
       <c r="F89" s="2"/>
       <c r="G89" s="2"/>
-      <c r="H89" s="110"/>
-      <c r="I89" s="110"/>
-      <c r="J89" s="110"/>
-      <c r="K89" s="110"/>
+      <c r="H89" s="115"/>
+      <c r="I89" s="115"/>
+      <c r="J89" s="115"/>
+      <c r="K89" s="115"/>
       <c r="L89" s="2"/>
     </row>
     <row r="90" spans="13:17" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
feat(requisiciones): máscara de caducidad, un libro por municipio, borde inferior y diálogo propio
- Caducidad: máscara DD-MM-AA al teclear (31 salta solo al mes, 06 al año, se detiene en 31-06-29;
  no admite dígitos de más; separadores a mano completan con ceros; JUL-29 se respeta) y, con la
  fecha completa, pasa sola a la cantidad.
- Exportación: cada municipio sale en UN archivo con una pestaña por unidad (las que tienen reparto)
  y la municipal al final; los hospitales, su sola hoja. Aplica al paquete .zip y al botón de cada
  municipio. Las pestañas son copias de la plantilla (logos, bordes y celdas combinadas) con su
  propia área de impresión.
- Plantilla: borde inferior del último biológico también en las celdas combinadas (A-F y K).
- Nombre de la entrega: diálogo propio de SIREVAQ (con sugerencias) en lugar del cuadro del navegador.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/requisiciones_plantilla.xlsx
+++ b/requisiciones_plantilla.xlsx
@@ -452,7 +452,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -783,30 +783,6 @@
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -855,7 +831,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="116">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -1051,22 +1027,10 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="12" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1154,7 +1118,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1166,7 +1130,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -1189,11 +1153,11 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1202,17 +1166,17 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1224,11 +1188,11 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -2708,519 +2672,519 @@
       <c r="L54" s="1"/>
     </row>
     <row r="55" ht="26.25" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="64"/>
-      <c r="B55" s="65"/>
-      <c r="C55" s="66"/>
-      <c r="D55" s="38"/>
-      <c r="E55" s="39"/>
-      <c r="F55" s="40"/>
+      <c r="A55" s="56"/>
+      <c r="B55" s="57"/>
+      <c r="C55" s="58"/>
+      <c r="D55" s="59"/>
+      <c r="E55" s="60"/>
+      <c r="F55" s="61"/>
       <c r="G55" s="47"/>
       <c r="H55" s="47"/>
       <c r="I55" s="48"/>
       <c r="J55" s="49"/>
-      <c r="K55" s="67"/>
+      <c r="K55" s="63"/>
       <c r="L55" s="1"/>
     </row>
     <row r="56" ht="25.5" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="68"/>
-      <c r="B56" s="69" t="s">
+      <c r="A56" s="64"/>
+      <c r="B56" s="65" t="s">
         <v>77</v>
       </c>
-      <c r="C56" s="69"/>
-      <c r="D56" s="69"/>
-      <c r="E56" s="69"/>
-      <c r="F56" s="69"/>
-      <c r="G56" s="69"/>
-      <c r="H56" s="69"/>
-      <c r="I56" s="69"/>
-      <c r="J56" s="69"/>
-      <c r="K56" s="70"/>
+      <c r="C56" s="65"/>
+      <c r="D56" s="65"/>
+      <c r="E56" s="65"/>
+      <c r="F56" s="65"/>
+      <c r="G56" s="65"/>
+      <c r="H56" s="65"/>
+      <c r="I56" s="65"/>
+      <c r="J56" s="65"/>
+      <c r="K56" s="66"/>
       <c r="L56" s="55"/>
     </row>
     <row r="57" ht="25.5" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="71"/>
-      <c r="B57" s="72"/>
-      <c r="C57" s="73"/>
-      <c r="D57" s="74"/>
-      <c r="E57" s="74"/>
-      <c r="F57" s="74"/>
-      <c r="G57" s="75"/>
-      <c r="H57" s="75"/>
-      <c r="I57" s="76"/>
-      <c r="J57" s="77"/>
-      <c r="K57" s="78"/>
+      <c r="A57" s="67"/>
+      <c r="B57" s="68"/>
+      <c r="C57" s="69"/>
+      <c r="D57" s="70"/>
+      <c r="E57" s="70"/>
+      <c r="F57" s="70"/>
+      <c r="G57" s="71"/>
+      <c r="H57" s="71"/>
+      <c r="I57" s="72"/>
+      <c r="J57" s="73"/>
+      <c r="K57" s="74"/>
       <c r="L57" s="8"/>
     </row>
     <row r="58" ht="25.5" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="71"/>
+      <c r="A58" s="67"/>
       <c r="B58" s="8"/>
-      <c r="C58" s="79" t="s">
+      <c r="C58" s="75" t="s">
         <v>78</v>
       </c>
-      <c r="D58" s="80"/>
-      <c r="E58" s="76"/>
-      <c r="F58" s="74"/>
-      <c r="G58" s="79" t="s">
+      <c r="D58" s="76"/>
+      <c r="E58" s="72"/>
+      <c r="F58" s="70"/>
+      <c r="G58" s="75" t="s">
         <v>79</v>
       </c>
-      <c r="H58" s="79"/>
-      <c r="I58" s="81"/>
-      <c r="J58" s="77"/>
-      <c r="K58" s="78"/>
+      <c r="H58" s="75"/>
+      <c r="I58" s="77"/>
+      <c r="J58" s="73"/>
+      <c r="K58" s="74"/>
       <c r="L58" s="8"/>
     </row>
     <row r="59" ht="25.5" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="71"/>
-      <c r="B59" s="72"/>
-      <c r="C59" s="73"/>
-      <c r="D59" s="74"/>
-      <c r="E59" s="74"/>
-      <c r="F59" s="74"/>
-      <c r="G59" s="75"/>
-      <c r="H59" s="75"/>
-      <c r="I59" s="76"/>
-      <c r="J59" s="77"/>
-      <c r="K59" s="78"/>
+      <c r="A59" s="67"/>
+      <c r="B59" s="68"/>
+      <c r="C59" s="69"/>
+      <c r="D59" s="70"/>
+      <c r="E59" s="70"/>
+      <c r="F59" s="70"/>
+      <c r="G59" s="71"/>
+      <c r="H59" s="71"/>
+      <c r="I59" s="72"/>
+      <c r="J59" s="73"/>
+      <c r="K59" s="74"/>
       <c r="L59" s="8"/>
     </row>
     <row r="60" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="82" t="s">
+      <c r="A60" s="78" t="s">
         <v>80</v>
       </c>
-      <c r="B60" s="82"/>
-      <c r="C60" s="82"/>
-      <c r="D60" s="82"/>
-      <c r="E60" s="82"/>
-      <c r="F60" s="82"/>
-      <c r="G60" s="82"/>
-      <c r="H60" s="82"/>
-      <c r="I60" s="82"/>
-      <c r="J60" s="82"/>
-      <c r="K60" s="82"/>
+      <c r="B60" s="78"/>
+      <c r="C60" s="78"/>
+      <c r="D60" s="78"/>
+      <c r="E60" s="78"/>
+      <c r="F60" s="78"/>
+      <c r="G60" s="78"/>
+      <c r="H60" s="78"/>
+      <c r="I60" s="78"/>
+      <c r="J60" s="78"/>
+      <c r="K60" s="78"/>
       <c r="L60" s="8"/>
     </row>
     <row r="61" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="83"/>
-      <c r="B61" s="84"/>
-      <c r="C61" s="84"/>
-      <c r="D61" s="84"/>
-      <c r="E61" s="84"/>
-      <c r="F61" s="84"/>
-      <c r="G61" s="84"/>
-      <c r="H61" s="84"/>
-      <c r="I61" s="84"/>
-      <c r="J61" s="84"/>
-      <c r="K61" s="85"/>
+      <c r="A61" s="79"/>
+      <c r="B61" s="80"/>
+      <c r="C61" s="80"/>
+      <c r="D61" s="80"/>
+      <c r="E61" s="80"/>
+      <c r="F61" s="80"/>
+      <c r="G61" s="80"/>
+      <c r="H61" s="80"/>
+      <c r="I61" s="80"/>
+      <c r="J61" s="80"/>
+      <c r="K61" s="81"/>
       <c r="L61" s="8"/>
     </row>
     <row r="62" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="83"/>
-      <c r="B62" s="84"/>
-      <c r="C62" s="84"/>
-      <c r="D62" s="84"/>
-      <c r="E62" s="84"/>
-      <c r="F62" s="84"/>
-      <c r="G62" s="84"/>
-      <c r="H62" s="84"/>
-      <c r="I62" s="84"/>
-      <c r="J62" s="84"/>
-      <c r="K62" s="83"/>
-      <c r="L62" s="83"/>
+      <c r="A62" s="79"/>
+      <c r="B62" s="80"/>
+      <c r="C62" s="80"/>
+      <c r="D62" s="80"/>
+      <c r="E62" s="80"/>
+      <c r="F62" s="80"/>
+      <c r="G62" s="80"/>
+      <c r="H62" s="80"/>
+      <c r="I62" s="80"/>
+      <c r="J62" s="80"/>
+      <c r="K62" s="79"/>
+      <c r="L62" s="79"/>
     </row>
     <row r="63" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="83"/>
-      <c r="B63" s="84"/>
-      <c r="C63" s="84"/>
-      <c r="D63" s="84"/>
-      <c r="E63" s="84"/>
-      <c r="F63" s="84"/>
-      <c r="G63" s="84"/>
-      <c r="H63" s="84"/>
-      <c r="I63" s="84"/>
-      <c r="J63" s="84"/>
-      <c r="K63" s="83"/>
-      <c r="L63" s="73"/>
+      <c r="A63" s="79"/>
+      <c r="B63" s="80"/>
+      <c r="C63" s="80"/>
+      <c r="D63" s="80"/>
+      <c r="E63" s="80"/>
+      <c r="F63" s="80"/>
+      <c r="G63" s="80"/>
+      <c r="H63" s="80"/>
+      <c r="I63" s="80"/>
+      <c r="J63" s="80"/>
+      <c r="K63" s="79"/>
+      <c r="L63" s="69"/>
     </row>
     <row r="64" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="86"/>
-      <c r="B64" s="87"/>
-      <c r="C64" s="88"/>
-      <c r="D64" s="88"/>
-      <c r="E64" s="88"/>
-      <c r="F64" s="87"/>
-      <c r="G64" s="87"/>
-      <c r="H64" s="87"/>
-      <c r="I64" s="88"/>
-      <c r="J64" s="88"/>
-      <c r="K64" s="88"/>
+      <c r="A64" s="82"/>
+      <c r="B64" s="83"/>
+      <c r="C64" s="84"/>
+      <c r="D64" s="84"/>
+      <c r="E64" s="84"/>
+      <c r="F64" s="83"/>
+      <c r="G64" s="83"/>
+      <c r="H64" s="83"/>
+      <c r="I64" s="84"/>
+      <c r="J64" s="84"/>
+      <c r="K64" s="84"/>
       <c r="L64" s="8"/>
     </row>
     <row r="65" ht="30" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="86"/>
-      <c r="B65" s="87"/>
-      <c r="C65" s="88"/>
-      <c r="D65" s="88"/>
-      <c r="E65" s="88"/>
-      <c r="F65" s="87"/>
+      <c r="A65" s="82"/>
+      <c r="B65" s="83"/>
+      <c r="C65" s="84"/>
+      <c r="D65" s="84"/>
+      <c r="E65" s="84"/>
+      <c r="F65" s="83"/>
       <c r="G65" s="8"/>
-      <c r="H65" s="87"/>
-      <c r="I65" s="87"/>
+      <c r="H65" s="83"/>
+      <c r="I65" s="83"/>
       <c r="J65" s="8"/>
       <c r="K65" s="8"/>
       <c r="L65" s="8"/>
     </row>
     <row r="66" ht="30" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="89"/>
-      <c r="B66" s="90"/>
-      <c r="C66" s="91"/>
-      <c r="D66" s="91"/>
-      <c r="E66" s="91"/>
-      <c r="F66" s="90"/>
-      <c r="G66" s="92"/>
-      <c r="H66" s="90"/>
-      <c r="I66" s="90"/>
-      <c r="J66" s="92"/>
-      <c r="K66" s="92"/>
+      <c r="A66" s="85"/>
+      <c r="B66" s="86"/>
+      <c r="C66" s="87"/>
+      <c r="D66" s="87"/>
+      <c r="E66" s="87"/>
+      <c r="F66" s="86"/>
+      <c r="G66" s="88"/>
+      <c r="H66" s="86"/>
+      <c r="I66" s="86"/>
+      <c r="J66" s="88"/>
+      <c r="K66" s="88"/>
       <c r="L66" s="8"/>
     </row>
     <row r="67" ht="19.5" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="93" t="s">
+      <c r="A67" s="89" t="s">
         <v>81</v>
       </c>
-      <c r="B67" s="93"/>
-      <c r="C67" s="93"/>
-      <c r="D67" s="94"/>
-      <c r="E67" s="94"/>
-      <c r="F67" s="95"/>
-      <c r="G67" s="96"/>
-      <c r="H67" s="97" t="s">
+      <c r="B67" s="89"/>
+      <c r="C67" s="89"/>
+      <c r="D67" s="90"/>
+      <c r="E67" s="90"/>
+      <c r="F67" s="91"/>
+      <c r="G67" s="92"/>
+      <c r="H67" s="93" t="s">
         <v>82</v>
       </c>
-      <c r="I67" s="97"/>
-      <c r="J67" s="97"/>
-      <c r="K67" s="97"/>
-      <c r="L67" s="98"/>
+      <c r="I67" s="93"/>
+      <c r="J67" s="93"/>
+      <c r="K67" s="93"/>
+      <c r="L67" s="94"/>
     </row>
     <row r="68" ht="20.1" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="95" t="s">
+      <c r="A68" s="91" t="s">
         <v>83</v>
       </c>
-      <c r="B68" s="95"/>
-      <c r="C68" s="95"/>
-      <c r="D68" s="95"/>
-      <c r="E68" s="95"/>
-      <c r="F68" s="95"/>
-      <c r="G68" s="96"/>
-      <c r="H68" s="95" t="s">
+      <c r="B68" s="91"/>
+      <c r="C68" s="91"/>
+      <c r="D68" s="91"/>
+      <c r="E68" s="91"/>
+      <c r="F68" s="91"/>
+      <c r="G68" s="92"/>
+      <c r="H68" s="91" t="s">
         <v>84</v>
       </c>
-      <c r="I68" s="95"/>
-      <c r="J68" s="95"/>
-      <c r="K68" s="95"/>
+      <c r="I68" s="91"/>
+      <c r="J68" s="91"/>
+      <c r="K68" s="91"/>
       <c r="L68" s="12"/>
     </row>
     <row r="69" ht="30" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="95"/>
-      <c r="B69" s="95"/>
-      <c r="C69" s="95"/>
-      <c r="D69" s="95"/>
-      <c r="E69" s="95"/>
-      <c r="F69" s="95"/>
-      <c r="G69" s="96"/>
-      <c r="H69" s="95"/>
-      <c r="I69" s="95"/>
-      <c r="J69" s="95"/>
-      <c r="K69" s="95"/>
+      <c r="A69" s="91"/>
+      <c r="B69" s="91"/>
+      <c r="C69" s="91"/>
+      <c r="D69" s="91"/>
+      <c r="E69" s="91"/>
+      <c r="F69" s="91"/>
+      <c r="G69" s="92"/>
+      <c r="H69" s="91"/>
+      <c r="I69" s="91"/>
+      <c r="J69" s="91"/>
+      <c r="K69" s="91"/>
       <c r="L69" s="12"/>
     </row>
     <row r="70" ht="30" customHeight="1" spans="1:17" s="12" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="95"/>
-      <c r="B70" s="95"/>
-      <c r="C70" s="95"/>
-      <c r="D70" s="95"/>
-      <c r="E70" s="95"/>
-      <c r="F70" s="95"/>
-      <c r="G70" s="96"/>
-      <c r="H70" s="95"/>
-      <c r="I70" s="95"/>
-      <c r="J70" s="95"/>
-      <c r="K70" s="95"/>
+      <c r="A70" s="91"/>
+      <c r="B70" s="91"/>
+      <c r="C70" s="91"/>
+      <c r="D70" s="91"/>
+      <c r="E70" s="91"/>
+      <c r="F70" s="91"/>
+      <c r="G70" s="92"/>
+      <c r="H70" s="91"/>
+      <c r="I70" s="91"/>
+      <c r="J70" s="91"/>
+      <c r="K70" s="91"/>
       <c r="L70" s="12"/>
     </row>
     <row r="71" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="95"/>
-      <c r="B71" s="95"/>
-      <c r="C71" s="95"/>
-      <c r="D71" s="95"/>
-      <c r="E71" s="95"/>
-      <c r="F71" s="95"/>
-      <c r="G71" s="96"/>
-      <c r="H71" s="95"/>
-      <c r="I71" s="95"/>
-      <c r="J71" s="95"/>
-      <c r="K71" s="95"/>
+      <c r="A71" s="91"/>
+      <c r="B71" s="91"/>
+      <c r="C71" s="91"/>
+      <c r="D71" s="91"/>
+      <c r="E71" s="91"/>
+      <c r="F71" s="91"/>
+      <c r="G71" s="92"/>
+      <c r="H71" s="91"/>
+      <c r="I71" s="91"/>
+      <c r="J71" s="91"/>
+      <c r="K71" s="91"/>
       <c r="L71" s="12"/>
     </row>
     <row r="72" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="95"/>
-      <c r="B72" s="95"/>
-      <c r="C72" s="96"/>
-      <c r="D72" s="96"/>
-      <c r="E72" s="96"/>
-      <c r="F72" s="95"/>
-      <c r="G72" s="96"/>
-      <c r="H72" s="95"/>
-      <c r="I72" s="95"/>
-      <c r="J72" s="96"/>
-      <c r="K72" s="96"/>
+      <c r="A72" s="91"/>
+      <c r="B72" s="91"/>
+      <c r="C72" s="92"/>
+      <c r="D72" s="92"/>
+      <c r="E72" s="92"/>
+      <c r="F72" s="91"/>
+      <c r="G72" s="92"/>
+      <c r="H72" s="91"/>
+      <c r="I72" s="91"/>
+      <c r="J72" s="92"/>
+      <c r="K72" s="92"/>
       <c r="L72" s="12"/>
     </row>
     <row r="73" ht="30" customHeight="1" spans="1:17" s="8" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="99"/>
-      <c r="B73" s="99"/>
-      <c r="C73" s="99"/>
-      <c r="D73" s="100"/>
-      <c r="E73" s="100"/>
-      <c r="F73" s="101"/>
-      <c r="G73" s="102"/>
-      <c r="H73" s="99"/>
-      <c r="I73" s="99"/>
-      <c r="J73" s="99"/>
-      <c r="K73" s="99"/>
-      <c r="L73" s="103"/>
+      <c r="A73" s="95"/>
+      <c r="B73" s="95"/>
+      <c r="C73" s="95"/>
+      <c r="D73" s="96"/>
+      <c r="E73" s="96"/>
+      <c r="F73" s="97"/>
+      <c r="G73" s="98"/>
+      <c r="H73" s="95"/>
+      <c r="I73" s="95"/>
+      <c r="J73" s="95"/>
+      <c r="K73" s="95"/>
+      <c r="L73" s="99"/>
     </row>
     <row r="74" ht="18.75" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="104" t="s">
+      <c r="A74" s="100" t="s">
         <v>85</v>
       </c>
-      <c r="B74" s="104"/>
-      <c r="C74" s="104"/>
-      <c r="D74" s="100"/>
-      <c r="E74" s="100"/>
-      <c r="F74" s="101"/>
-      <c r="G74" s="102"/>
-      <c r="H74" s="95" t="s">
+      <c r="B74" s="100"/>
+      <c r="C74" s="100"/>
+      <c r="D74" s="96"/>
+      <c r="E74" s="96"/>
+      <c r="F74" s="97"/>
+      <c r="G74" s="98"/>
+      <c r="H74" s="91" t="s">
         <v>86</v>
       </c>
-      <c r="I74" s="95"/>
-      <c r="J74" s="95"/>
-      <c r="K74" s="95"/>
+      <c r="I74" s="91"/>
+      <c r="J74" s="91"/>
+      <c r="K74" s="91"/>
       <c r="L74" s="8"/>
     </row>
     <row r="75" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="95" t="s">
+      <c r="A75" s="91" t="s">
         <v>87</v>
       </c>
-      <c r="B75" s="95"/>
-      <c r="C75" s="95"/>
-      <c r="D75" s="95"/>
-      <c r="E75" s="95"/>
-      <c r="F75" s="94"/>
-      <c r="G75" s="100"/>
-      <c r="H75" s="94" t="s">
+      <c r="B75" s="91"/>
+      <c r="C75" s="91"/>
+      <c r="D75" s="91"/>
+      <c r="E75" s="91"/>
+      <c r="F75" s="90"/>
+      <c r="G75" s="96"/>
+      <c r="H75" s="90" t="s">
         <v>88</v>
       </c>
-      <c r="I75" s="94"/>
-      <c r="J75" s="94"/>
-      <c r="K75" s="94"/>
-      <c r="L75" s="103"/>
+      <c r="I75" s="90"/>
+      <c r="J75" s="90"/>
+      <c r="K75" s="90"/>
+      <c r="L75" s="99"/>
     </row>
     <row r="76" ht="20.25" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="105"/>
-      <c r="B76" s="105"/>
-      <c r="C76" s="105"/>
-      <c r="D76" s="90"/>
-      <c r="E76" s="90"/>
-      <c r="F76" s="106"/>
-      <c r="G76" s="107"/>
-      <c r="H76" s="108"/>
-      <c r="I76" s="108"/>
-      <c r="J76" s="108"/>
-      <c r="K76" s="109"/>
-      <c r="L76" s="110"/>
+      <c r="A76" s="101"/>
+      <c r="B76" s="101"/>
+      <c r="C76" s="101"/>
+      <c r="D76" s="86"/>
+      <c r="E76" s="86"/>
+      <c r="F76" s="102"/>
+      <c r="G76" s="103"/>
+      <c r="H76" s="104"/>
+      <c r="I76" s="104"/>
+      <c r="J76" s="104"/>
+      <c r="K76" s="105"/>
+      <c r="L76" s="106"/>
     </row>
     <row r="77" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="111"/>
-      <c r="B77" s="111"/>
-      <c r="C77" s="111"/>
-      <c r="D77" s="112"/>
-      <c r="E77" s="112"/>
+      <c r="A77" s="107"/>
+      <c r="B77" s="107"/>
+      <c r="C77" s="107"/>
+      <c r="D77" s="108"/>
+      <c r="E77" s="108"/>
       <c r="F77" s="2"/>
-      <c r="G77" s="113"/>
-      <c r="H77" s="114" t="s">
+      <c r="G77" s="109"/>
+      <c r="H77" s="110" t="s">
         <v>89</v>
       </c>
-      <c r="I77" s="115"/>
-      <c r="J77" s="115"/>
-      <c r="K77" s="115"/>
+      <c r="I77" s="111"/>
+      <c r="J77" s="111"/>
+      <c r="K77" s="111"/>
       <c r="L77" s="2"/>
     </row>
     <row r="78" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="111"/>
-      <c r="B78" s="111"/>
-      <c r="C78" s="111"/>
+      <c r="A78" s="107"/>
+      <c r="B78" s="107"/>
+      <c r="C78" s="107"/>
       <c r="D78" s="2"/>
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
-      <c r="G78" s="113"/>
-      <c r="H78" s="115"/>
-      <c r="I78" s="115"/>
-      <c r="J78" s="115"/>
-      <c r="K78" s="115"/>
+      <c r="G78" s="109"/>
+      <c r="H78" s="111"/>
+      <c r="I78" s="111"/>
+      <c r="J78" s="111"/>
+      <c r="K78" s="111"/>
       <c r="L78" s="2"/>
     </row>
     <row r="79" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="111"/>
-      <c r="B79" s="111"/>
-      <c r="C79" s="111"/>
+      <c r="A79" s="107"/>
+      <c r="B79" s="107"/>
+      <c r="C79" s="107"/>
       <c r="D79" s="2"/>
       <c r="E79" s="2"/>
       <c r="F79" s="2"/>
-      <c r="G79" s="113"/>
-      <c r="H79" s="115"/>
-      <c r="I79" s="115"/>
-      <c r="J79" s="115"/>
-      <c r="K79" s="115"/>
+      <c r="G79" s="109"/>
+      <c r="H79" s="111"/>
+      <c r="I79" s="111"/>
+      <c r="J79" s="111"/>
+      <c r="K79" s="111"/>
       <c r="L79" s="2"/>
     </row>
     <row r="80" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="111"/>
-      <c r="B80" s="111"/>
-      <c r="C80" s="111"/>
+      <c r="A80" s="107"/>
+      <c r="B80" s="107"/>
+      <c r="C80" s="107"/>
       <c r="D80" s="2"/>
       <c r="E80" s="2"/>
       <c r="F80" s="2"/>
-      <c r="G80" s="113"/>
-      <c r="H80" s="115"/>
-      <c r="I80" s="115"/>
-      <c r="J80" s="115"/>
-      <c r="K80" s="115"/>
+      <c r="G80" s="109"/>
+      <c r="H80" s="111"/>
+      <c r="I80" s="111"/>
+      <c r="J80" s="111"/>
+      <c r="K80" s="111"/>
       <c r="L80" s="2"/>
     </row>
     <row r="81" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="111"/>
-      <c r="B81" s="111"/>
-      <c r="C81" s="111"/>
+      <c r="A81" s="107"/>
+      <c r="B81" s="107"/>
+      <c r="C81" s="107"/>
       <c r="D81" s="2"/>
       <c r="E81" s="2"/>
       <c r="F81" s="2"/>
-      <c r="G81" s="113"/>
-      <c r="H81" s="115"/>
-      <c r="I81" s="115"/>
-      <c r="J81" s="115"/>
-      <c r="K81" s="115"/>
+      <c r="G81" s="109"/>
+      <c r="H81" s="111"/>
+      <c r="I81" s="111"/>
+      <c r="J81" s="111"/>
+      <c r="K81" s="111"/>
       <c r="L81" s="2"/>
     </row>
     <row r="82" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="111"/>
-      <c r="B82" s="111"/>
-      <c r="C82" s="111"/>
+      <c r="A82" s="107"/>
+      <c r="B82" s="107"/>
+      <c r="C82" s="107"/>
       <c r="D82" s="2"/>
       <c r="E82" s="2"/>
       <c r="F82" s="2"/>
-      <c r="G82" s="113"/>
-      <c r="H82" s="115"/>
-      <c r="I82" s="115"/>
-      <c r="J82" s="115"/>
-      <c r="K82" s="115"/>
+      <c r="G82" s="109"/>
+      <c r="H82" s="111"/>
+      <c r="I82" s="111"/>
+      <c r="J82" s="111"/>
+      <c r="K82" s="111"/>
       <c r="L82" s="2"/>
     </row>
     <row r="83" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="111"/>
-      <c r="B83" s="111"/>
-      <c r="C83" s="111"/>
+      <c r="A83" s="107"/>
+      <c r="B83" s="107"/>
+      <c r="C83" s="107"/>
       <c r="D83" s="2"/>
       <c r="E83" s="2"/>
       <c r="F83" s="2"/>
-      <c r="G83" s="113"/>
-      <c r="H83" s="115"/>
-      <c r="I83" s="115"/>
-      <c r="J83" s="115"/>
-      <c r="K83" s="115"/>
+      <c r="G83" s="109"/>
+      <c r="H83" s="111"/>
+      <c r="I83" s="111"/>
+      <c r="J83" s="111"/>
+      <c r="K83" s="111"/>
       <c r="L83" s="2"/>
     </row>
     <row r="84" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="111"/>
-      <c r="B84" s="111"/>
-      <c r="C84" s="111"/>
+      <c r="A84" s="107"/>
+      <c r="B84" s="107"/>
+      <c r="C84" s="107"/>
       <c r="D84" s="2"/>
       <c r="E84" s="2"/>
       <c r="F84" s="2"/>
-      <c r="G84" s="113"/>
-      <c r="H84" s="115"/>
-      <c r="I84" s="115"/>
-      <c r="J84" s="115"/>
-      <c r="K84" s="115"/>
+      <c r="G84" s="109"/>
+      <c r="H84" s="111"/>
+      <c r="I84" s="111"/>
+      <c r="J84" s="111"/>
+      <c r="K84" s="111"/>
       <c r="L84" s="2"/>
     </row>
     <row r="85" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="111"/>
-      <c r="B85" s="111"/>
-      <c r="C85" s="111"/>
+      <c r="A85" s="107"/>
+      <c r="B85" s="107"/>
+      <c r="C85" s="107"/>
       <c r="D85" s="2"/>
       <c r="E85" s="2"/>
       <c r="F85" s="2"/>
-      <c r="G85" s="113"/>
-      <c r="H85" s="115"/>
-      <c r="I85" s="115"/>
-      <c r="J85" s="115"/>
-      <c r="K85" s="115"/>
+      <c r="G85" s="109"/>
+      <c r="H85" s="111"/>
+      <c r="I85" s="111"/>
+      <c r="J85" s="111"/>
+      <c r="K85" s="111"/>
       <c r="L85" s="2"/>
     </row>
     <row r="86" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="111"/>
-      <c r="B86" s="111"/>
-      <c r="C86" s="111"/>
+      <c r="A86" s="107"/>
+      <c r="B86" s="107"/>
+      <c r="C86" s="107"/>
       <c r="D86" s="2"/>
       <c r="E86" s="2"/>
       <c r="F86" s="2"/>
-      <c r="G86" s="113"/>
-      <c r="H86" s="115"/>
-      <c r="I86" s="115"/>
-      <c r="J86" s="115"/>
-      <c r="K86" s="115"/>
+      <c r="G86" s="109"/>
+      <c r="H86" s="111"/>
+      <c r="I86" s="111"/>
+      <c r="J86" s="111"/>
+      <c r="K86" s="111"/>
       <c r="L86" s="2"/>
     </row>
     <row r="87" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="111"/>
-      <c r="B87" s="111"/>
-      <c r="C87" s="111"/>
+      <c r="A87" s="107"/>
+      <c r="B87" s="107"/>
+      <c r="C87" s="107"/>
       <c r="D87" s="2"/>
       <c r="E87" s="2"/>
       <c r="F87" s="2"/>
-      <c r="G87" s="113"/>
-      <c r="H87" s="115"/>
-      <c r="I87" s="115"/>
-      <c r="J87" s="115"/>
-      <c r="K87" s="115"/>
+      <c r="G87" s="109"/>
+      <c r="H87" s="111"/>
+      <c r="I87" s="111"/>
+      <c r="J87" s="111"/>
+      <c r="K87" s="111"/>
       <c r="L87" s="2"/>
     </row>
     <row r="88" ht="30" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A88" s="111"/>
-      <c r="B88" s="111"/>
-      <c r="C88" s="111"/>
+      <c r="A88" s="107"/>
+      <c r="B88" s="107"/>
+      <c r="C88" s="107"/>
       <c r="D88" s="2"/>
       <c r="E88" s="2"/>
       <c r="F88" s="2"/>
-      <c r="G88" s="113"/>
-      <c r="H88" s="115"/>
-      <c r="I88" s="115"/>
-      <c r="J88" s="115"/>
-      <c r="K88" s="115"/>
+      <c r="G88" s="109"/>
+      <c r="H88" s="111"/>
+      <c r="I88" s="111"/>
+      <c r="J88" s="111"/>
+      <c r="K88" s="111"/>
       <c r="L88" s="2"/>
     </row>
     <row r="89" ht="30" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A89" s="111"/>
-      <c r="B89" s="111"/>
-      <c r="C89" s="111"/>
+      <c r="A89" s="107"/>
+      <c r="B89" s="107"/>
+      <c r="C89" s="107"/>
       <c r="D89" s="2"/>
       <c r="E89" s="2"/>
       <c r="F89" s="2"/>
       <c r="G89" s="2"/>
-      <c r="H89" s="115"/>
-      <c r="I89" s="115"/>
-      <c r="J89" s="115"/>
-      <c r="K89" s="115"/>
+      <c r="H89" s="111"/>
+      <c r="I89" s="111"/>
+      <c r="J89" s="111"/>
+      <c r="K89" s="111"/>
       <c r="L89" s="2"/>
     </row>
     <row r="90" spans="13:17" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
fix(requisiciones): caducidad con día en el Excel y sello de unidad como cuadro de texto
- La caducidad con día distinto del último del mes sale completa (27-AGO-29); sin día sigue AGO-29.
- "SELLO UNIDAD" vuelve a ser un cuadro de texto #F9F9F9 como en el formato original (como texto de
  celda salía casi negro en impresoras de tóner). Solo va en unidad y hospitales.
- La plantilla se pide sin caché.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/requisiciones_plantilla.xlsx
+++ b/requisiciones_plantilla.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="89">
   <si>
     <t>SERVICIOS DE SALUD DEL ESTADO DE QUERÉTARO</t>
   </si>
@@ -295,10 +295,6 @@
   <si>
     <t>RECIBE: NOMBRE COMPLETO Y FIRMA</t>
   </si>
-  <si>
-    <t xml:space="preserve">SELLO
-UNIDAD</t>
-  </si>
 </sst>
 </file>
 
@@ -309,7 +305,7 @@
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy;@"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -420,11 +416,6 @@
       <sz val="10"/>
       <name val="Arial Nova"/>
     </font>
-    <font>
-      <color rgb="FFF9F9F9"/>
-      <sz val="138"/>
-      <name val="Arial"/>
-    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -831,7 +822,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -1186,10 +1177,6 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -3011,12 +2998,10 @@
       <c r="E77" s="108"/>
       <c r="F77" s="2"/>
       <c r="G77" s="109"/>
-      <c r="H77" s="110" t="s">
-        <v>89</v>
-      </c>
-      <c r="I77" s="111"/>
-      <c r="J77" s="111"/>
-      <c r="K77" s="111"/>
+      <c r="H77" s="110"/>
+      <c r="I77" s="110"/>
+      <c r="J77" s="110"/>
+      <c r="K77" s="110"/>
       <c r="L77" s="2"/>
     </row>
     <row r="78" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3027,10 +3012,10 @@
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
       <c r="G78" s="109"/>
-      <c r="H78" s="111"/>
-      <c r="I78" s="111"/>
-      <c r="J78" s="111"/>
-      <c r="K78" s="111"/>
+      <c r="H78" s="110"/>
+      <c r="I78" s="110"/>
+      <c r="J78" s="110"/>
+      <c r="K78" s="110"/>
       <c r="L78" s="2"/>
     </row>
     <row r="79" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3041,10 +3026,10 @@
       <c r="E79" s="2"/>
       <c r="F79" s="2"/>
       <c r="G79" s="109"/>
-      <c r="H79" s="111"/>
-      <c r="I79" s="111"/>
-      <c r="J79" s="111"/>
-      <c r="K79" s="111"/>
+      <c r="H79" s="110"/>
+      <c r="I79" s="110"/>
+      <c r="J79" s="110"/>
+      <c r="K79" s="110"/>
       <c r="L79" s="2"/>
     </row>
     <row r="80" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3055,10 +3040,10 @@
       <c r="E80" s="2"/>
       <c r="F80" s="2"/>
       <c r="G80" s="109"/>
-      <c r="H80" s="111"/>
-      <c r="I80" s="111"/>
-      <c r="J80" s="111"/>
-      <c r="K80" s="111"/>
+      <c r="H80" s="110"/>
+      <c r="I80" s="110"/>
+      <c r="J80" s="110"/>
+      <c r="K80" s="110"/>
       <c r="L80" s="2"/>
     </row>
     <row r="81" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3069,10 +3054,10 @@
       <c r="E81" s="2"/>
       <c r="F81" s="2"/>
       <c r="G81" s="109"/>
-      <c r="H81" s="111"/>
-      <c r="I81" s="111"/>
-      <c r="J81" s="111"/>
-      <c r="K81" s="111"/>
+      <c r="H81" s="110"/>
+      <c r="I81" s="110"/>
+      <c r="J81" s="110"/>
+      <c r="K81" s="110"/>
       <c r="L81" s="2"/>
     </row>
     <row r="82" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3083,10 +3068,10 @@
       <c r="E82" s="2"/>
       <c r="F82" s="2"/>
       <c r="G82" s="109"/>
-      <c r="H82" s="111"/>
-      <c r="I82" s="111"/>
-      <c r="J82" s="111"/>
-      <c r="K82" s="111"/>
+      <c r="H82" s="110"/>
+      <c r="I82" s="110"/>
+      <c r="J82" s="110"/>
+      <c r="K82" s="110"/>
       <c r="L82" s="2"/>
     </row>
     <row r="83" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3097,10 +3082,10 @@
       <c r="E83" s="2"/>
       <c r="F83" s="2"/>
       <c r="G83" s="109"/>
-      <c r="H83" s="111"/>
-      <c r="I83" s="111"/>
-      <c r="J83" s="111"/>
-      <c r="K83" s="111"/>
+      <c r="H83" s="110"/>
+      <c r="I83" s="110"/>
+      <c r="J83" s="110"/>
+      <c r="K83" s="110"/>
       <c r="L83" s="2"/>
     </row>
     <row r="84" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3111,10 +3096,10 @@
       <c r="E84" s="2"/>
       <c r="F84" s="2"/>
       <c r="G84" s="109"/>
-      <c r="H84" s="111"/>
-      <c r="I84" s="111"/>
-      <c r="J84" s="111"/>
-      <c r="K84" s="111"/>
+      <c r="H84" s="110"/>
+      <c r="I84" s="110"/>
+      <c r="J84" s="110"/>
+      <c r="K84" s="110"/>
       <c r="L84" s="2"/>
     </row>
     <row r="85" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3125,10 +3110,10 @@
       <c r="E85" s="2"/>
       <c r="F85" s="2"/>
       <c r="G85" s="109"/>
-      <c r="H85" s="111"/>
-      <c r="I85" s="111"/>
-      <c r="J85" s="111"/>
-      <c r="K85" s="111"/>
+      <c r="H85" s="110"/>
+      <c r="I85" s="110"/>
+      <c r="J85" s="110"/>
+      <c r="K85" s="110"/>
       <c r="L85" s="2"/>
     </row>
     <row r="86" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3139,10 +3124,10 @@
       <c r="E86" s="2"/>
       <c r="F86" s="2"/>
       <c r="G86" s="109"/>
-      <c r="H86" s="111"/>
-      <c r="I86" s="111"/>
-      <c r="J86" s="111"/>
-      <c r="K86" s="111"/>
+      <c r="H86" s="110"/>
+      <c r="I86" s="110"/>
+      <c r="J86" s="110"/>
+      <c r="K86" s="110"/>
       <c r="L86" s="2"/>
     </row>
     <row r="87" ht="30" customHeight="1" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3153,10 +3138,10 @@
       <c r="E87" s="2"/>
       <c r="F87" s="2"/>
       <c r="G87" s="109"/>
-      <c r="H87" s="111"/>
-      <c r="I87" s="111"/>
-      <c r="J87" s="111"/>
-      <c r="K87" s="111"/>
+      <c r="H87" s="110"/>
+      <c r="I87" s="110"/>
+      <c r="J87" s="110"/>
+      <c r="K87" s="110"/>
       <c r="L87" s="2"/>
     </row>
     <row r="88" ht="30" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
@@ -3167,10 +3152,10 @@
       <c r="E88" s="2"/>
       <c r="F88" s="2"/>
       <c r="G88" s="109"/>
-      <c r="H88" s="111"/>
-      <c r="I88" s="111"/>
-      <c r="J88" s="111"/>
-      <c r="K88" s="111"/>
+      <c r="H88" s="110"/>
+      <c r="I88" s="110"/>
+      <c r="J88" s="110"/>
+      <c r="K88" s="110"/>
       <c r="L88" s="2"/>
     </row>
     <row r="89" ht="30" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
@@ -3181,10 +3166,10 @@
       <c r="E89" s="2"/>
       <c r="F89" s="2"/>
       <c r="G89" s="2"/>
-      <c r="H89" s="111"/>
-      <c r="I89" s="111"/>
-      <c r="J89" s="111"/>
-      <c r="K89" s="111"/>
+      <c r="H89" s="110"/>
+      <c r="I89" s="110"/>
+      <c r="J89" s="110"/>
+      <c r="K89" s="110"/>
       <c r="L89" s="2"/>
     </row>
     <row r="90" spans="13:17" x14ac:dyDescent="0.25"/>

</xml_diff>